<commit_message>
Clarify Parametres: show Calcul_A and Calcul_B WSEmax side by side
WSEmax is Vmax read on the survey stage-storage curve; Parametres now
lists Vmax/WSEmax/HW for both Method A and Method B with a short how-to.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -147,7 +147,6 @@
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,6 +166,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1338,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1656,25 +1656,30 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Résultats (formules — feuille Calcul_A)</t>
+          <t>Résultats Méthode A — Qout constant (feuille Calcul_A)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Vmax (m³)</t>
+          <t>Vmax_A (m³)</t>
         </is>
       </c>
       <c r="B27" s="18">
         <f>Calcul_A!B3</f>
         <v/>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Volume max stocké avec Qout fixe (Parametres B22)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>V_dimensionnement = Vmax × facteur (m³)</t>
+          <t>V_dimensionnement_A = Vmax_A × facteur (m³)</t>
         </is>
       </c>
       <c r="B28" s="18">
@@ -1685,7 +1690,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hmax approx (m) = Vmax / Aire</t>
+          <t>Hmax approx_A (m) = Vmax_A / Aire</t>
         </is>
       </c>
       <c r="B29" s="19">
@@ -1694,14 +1699,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Estimation grossière si l'aire de bassin est constante</t>
+          <t>Estimation grossière si l'aire de bassin est constante (pas le levé)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WSEmax depuis levé (m) — feuille Stage_Storage</t>
+          <t>WSEmax_A depuis levé (m) — feuille Stage_Storage</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -1710,14 +1715,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Niveau d'eau max lu sur courbe volume–cote du levé (recommandé)</t>
+          <t>Cote d'eau max pour le Vmax_A: on lit sur Stage_Storage quelle WSE donne ce volume (courbe volume–cote du levé)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HW max = WSEmax − radier Ø900 (m)</t>
+          <t>HW max_A = WSEmax_A − radier Ø900 (m)</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -1733,165 +1738,246 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Inlet control vs outlet control — qu'est-ce que ça veut dire?</t>
+          <t>Résultats Méthode B — Qout = f(H) FHWA (feuille Calcul_B)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>• Inlet control (contrôle à l'entrée): le débit est limité par l'entrée du ponceau (forme d'entrée, HW/D).</t>
+          <t>Vmax_B (m³)</t>
+        </is>
+      </c>
+      <c r="B34" s="18">
+        <f>Calcul_B!B7</f>
+        <v/>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Volume max stocké avec Q lu sur Courbe_QH_900 (dépend de Aire B24)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Le tuyau aval « n'aspire » pas assez pour influencer — Q dépend surtout de la charge amont H, pas de L ni de n.</t>
-        </is>
+          <t>V_dimensionnement_B = Vmax_B × facteur (m³)</t>
+        </is>
+      </c>
+      <c r="B35" s="18">
+        <f>B34*B23</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>• Outlet control (contrôle à la sortie / frottement): le débit dépend de la longueur, de n, de la pente et de la charge</t>
+          <t>WSEmax_B depuis levé (m) — feuille Stage_Storage</t>
+        </is>
+      </c>
+      <c r="B36" s="20">
+        <f>IF(B34&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B34&gt;=Stage_Storage!E18,"Hors table (&gt;=39.5 m — étendre levé)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B34,Stage_Storage!$E$11:$E$18,1))+(B34-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B34,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B34,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B34,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B34,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B34,Stage_Storage!$E$11:$E$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Même lecture volume→cote que B30, mais avec Vmax_B au lieu de Vmax_A</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (énergie amont → aval). Manning pleine section est une hypothèse de type outlet/frottement à section pleine.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>• Ici L/D = 56 (tuyau assez long) → le contrôle par frottement (outlet) est souvent plausible,</t>
+          <t>HW max_B = WSEmax_B − radier Ø900 (m)</t>
+        </is>
+      </c>
+      <c r="B37" s="20">
+        <f>IF(ISNUMBER(B36),B36-34.88,"")</f>
+        <v/>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Comparer à 2.40 m (limite patron)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  mais sans analyse FHWA/HY-8 on ne peut pas l'affirmer. Pour dimensionner la rétention, Q_plein constant est</t>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Comment lire WSEmax (A ou B)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  en général prudent (si la charge monte, le débit réel peut être un peu plus élevé → Vmax un peu plus bas).</t>
+          <t>1) Calcul_A (ou B) donne un volume max stocké Vmax pendant l'orage.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>• On n'a pas besoin de trancher IC/OC pour utiliser ce classeur: garder Qout = Q_plein (ou 1.77) suffit pour une 1re estimation.</t>
+          <t>2) La feuille Stage_Storage convertit vos surfaces de levé en courbe: volume cumulé ↔ cote d'eau (WSE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>3) WSEmax = la cote sur cette courbe qui correspond à ce Vmax (interpolation).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Exemple: si Vmax_A ≈ volume entre 37.28 m et 39.5 m sur le levé → WSEmax_A ≈ 38.75 m.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (n=0,013). Pas un jugement IC/OC complet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>• Le stockage commence quand Qin dépasse Qout; Vmax = max du volume stocké (pas (Qp−Qout)×durée).</t>
+          <t>4) Ce n'est PAS une cote saisie à la main: c'est Vmax lu sur le levé. Hmax≈V/Aire (B29) est plus grossier.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>• Méthode B: Qout = f(H) depuis feuille Courbe_QH_900 (FHWA inlet+outlet).</t>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Inlet control vs outlet control — qu'est-ce que ça veut dire?</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• Voir feuille Fichiers_lies pour les anciens Excel HY-8 / ponceau+fossé.</t>
+          <t>• Inlet control (contrôle à l'entrée): le débit est limité par l'entrée du ponceau (forme d'entrée, HW/D).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>• Vérifier que le radier amont Ø900 (34.88) est bien le fond de la zone de rétention étudiée.</t>
+          <t xml:space="preserve">  Le tuyau aval « n'aspire » pas assez pour influencer — Q dépend surtout de la charge amont H, pas de L ni de n.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>• Niveau max (WSEmax): feuille Stage_Storage + case Parametres!B30 (Vmax → cote du levé).</t>
+          <t>• Outlet control (contrôle à la sortie / frottement): le débit dépend de la longueur, de n, de la pente et de la charge</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Vmax_B courbe FHWA (m³)</t>
-        </is>
-      </c>
-      <c r="B50" s="18">
-        <f>Calcul_B!B7</f>
-        <v/>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Routage avec Q=f(H) — dépend de Aire_bassin (B24)</t>
+          <t xml:space="preserve">  (énergie amont → aval). Manning pleine section est une hypothèse de type outlet/frottement à section pleine.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>WSEmax (rappel)</t>
-        </is>
-      </c>
-      <c r="B51" s="21">
-        <f>B30</f>
-        <v/>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Même valeur que B30 — niveau max depuis levé Stage_Storage</t>
+          <t>• Ici L/D = 56 (tuyau assez long) → le contrôle par frottement (outlet) est souvent plausible,</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mais sans analyse FHWA/HY-8 on ne peut pas l'affirmer. Pour dimensionner la rétention, Q_plein constant est</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  en général prudent (si la charge monte, le débit réel peut être un peu plus élevé → Vmax un peu plus bas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>• On n'a pas besoin de trancher IC/OC pour utiliser ce classeur: garder Qout = Q_plein (ou 1.77) suffit pour une 1re estimation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (n=0,013). Pas un jugement IC/OC complet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>• Le stockage commence quand Qin dépasse Qout; Vmax = max du volume stocké (pas (Qp−Qout)×durée).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>• Méthode B: Qout = f(H) depuis feuille Courbe_QH_900 (FHWA inlet+outlet) — résultats en B34–B37.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>• Voir feuille Fichiers_lies pour les anciens Excel HY-8 / ponceau+fossé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>• Vérifier que le radier amont Ø900 (34.88) est bien le fond de la zone de rétention étudiée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>• WSEmax_A = B30 (depuis Vmax_A); WSEmax_B = B36 (depuis Vmax_B); les deux lisent Stage_Storage.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="21">
     <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A9:H10"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A58:H58"/>
     <mergeCell ref="A40:H40"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1913,7 +1999,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Hydrogramme d'entrée (point Ø1500 / entrée rétention) — FORMULES LIVE</t>
         </is>
@@ -1948,7 +2034,7 @@
           <t>t pointe (min)</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="22" t="n">
         <v>22.5</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1980,10 +2066,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="n">
+      <c r="A8" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="24" t="n">
         <v>0.081042</v>
       </c>
       <c r="C8" s="5">
@@ -1997,10 +2083,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="n">
+      <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="25" t="n">
+      <c r="B9" s="24" t="n">
         <v>0.121875</v>
       </c>
       <c r="C9" s="5">
@@ -2010,10 +2096,10 @@
       <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="n">
+      <c r="A10" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="24" t="n">
         <v>0.193438</v>
       </c>
       <c r="C10" s="5">
@@ -2023,10 +2109,10 @@
       <c r="D10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="n">
+      <c r="A11" s="23" t="n">
         <v>15</v>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="24" t="n">
         <v>0.333542</v>
       </c>
       <c r="C11" s="5">
@@ -2036,10 +2122,10 @@
       <c r="D11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="n">
+      <c r="A12" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="24" t="n">
         <v>0.657188</v>
       </c>
       <c r="C12" s="5">
@@ -2049,10 +2135,10 @@
       <c r="D12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="n">
+      <c r="A13" s="23" t="n">
         <v>22.5</v>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="8">
@@ -2066,10 +2152,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="n">
+      <c r="A14" s="23" t="n">
         <v>27.5</v>
       </c>
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="24" t="n">
         <v>0.608958</v>
       </c>
       <c r="C14" s="5">
@@ -2079,10 +2165,10 @@
       <c r="D14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="23" t="n">
         <v>32.5</v>
       </c>
-      <c r="B15" s="25" t="n">
+      <c r="B15" s="24" t="n">
         <v>0.401771</v>
       </c>
       <c r="C15" s="5">
@@ -2092,10 +2178,10 @@
       <c r="D15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="n">
+      <c r="A16" s="23" t="n">
         <v>37.5</v>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="24" t="n">
         <v>0.280104</v>
       </c>
       <c r="C16" s="5">
@@ -2105,10 +2191,10 @@
       <c r="D16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="24" t="n">
+      <c r="A17" s="23" t="n">
         <v>42.5</v>
       </c>
-      <c r="B17" s="25" t="n">
+      <c r="B17" s="24" t="n">
         <v>0.203438</v>
       </c>
       <c r="C17" s="5">
@@ -2118,10 +2204,10 @@
       <c r="D17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="24" t="n">
+      <c r="A18" s="23" t="n">
         <v>47.5</v>
       </c>
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="24" t="n">
         <v>0.152292</v>
       </c>
       <c r="C18" s="5">
@@ -2131,10 +2217,10 @@
       <c r="D18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="n">
+      <c r="A19" s="23" t="n">
         <v>52.5</v>
       </c>
-      <c r="B19" s="25" t="n">
+      <c r="B19" s="24" t="n">
         <v>0.116771</v>
       </c>
       <c r="C19" s="5">
@@ -2144,10 +2230,10 @@
       <c r="D19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="n">
+      <c r="A20" s="23" t="n">
         <v>57.5</v>
       </c>
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="24" t="n">
         <v>0.091146</v>
       </c>
       <c r="C20" s="5">
@@ -2162,7 +2248,7 @@
           <t>Qin max (contrôle)</t>
         </is>
       </c>
-      <c r="B22" s="26">
+      <c r="B22" s="25">
         <f>MAX(C8:C20)</f>
         <v/>
       </c>
@@ -2213,7 +2299,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Méthode A — Qout constant = capacité Ø900</t>
         </is>
@@ -2225,7 +2311,7 @@
           <t>Qout (m³/s)</t>
         </is>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="26">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -2236,7 +2322,7 @@
           <t>Vmax (m³)</t>
         </is>
       </c>
-      <c r="B3" s="28">
+      <c r="B3" s="27">
         <f>MAX(H8:H20)</f>
         <v/>
       </c>
@@ -2318,7 +2404,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24">
+      <c r="A8" s="23">
         <f>Hydrogramme!A8</f>
         <v/>
       </c>
@@ -2326,7 +2412,7 @@
         <f>Hydrogramme!C8</f>
         <v/>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2343,7 +2429,7 @@
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="29" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="4">
@@ -2352,7 +2438,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24">
+      <c r="A9" s="23">
         <f>Hydrogramme!A9</f>
         <v/>
       </c>
@@ -2360,7 +2446,7 @@
         <f>Hydrogramme!C9</f>
         <v/>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2368,19 +2454,19 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="23">
         <f>(A9-A8)*60</f>
         <v/>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="23">
         <f>0.5*(B8+B9)*E9</f>
         <v/>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="23">
         <f>F9-(H9-H8)</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="30">
         <f>MAX(0,H8+0.5*(D8+D9)*E9)</f>
         <v/>
       </c>
@@ -2390,7 +2476,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24">
+      <c r="A10" s="23">
         <f>Hydrogramme!A10</f>
         <v/>
       </c>
@@ -2398,7 +2484,7 @@
         <f>Hydrogramme!C10</f>
         <v/>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2406,19 +2492,19 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="23">
         <f>(A10-A9)*60</f>
         <v/>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="23">
         <f>0.5*(B9+B10)*E10</f>
         <v/>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="23">
         <f>F10-(H10-H9)</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="30">
         <f>MAX(0,H9+0.5*(D9+D10)*E10)</f>
         <v/>
       </c>
@@ -2428,7 +2514,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24">
+      <c r="A11" s="23">
         <f>Hydrogramme!A11</f>
         <v/>
       </c>
@@ -2436,7 +2522,7 @@
         <f>Hydrogramme!C11</f>
         <v/>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2444,19 +2530,19 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="23">
         <f>(A11-A10)*60</f>
         <v/>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="23">
         <f>0.5*(B10+B11)*E11</f>
         <v/>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="23">
         <f>F11-(H11-H10)</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="30">
         <f>MAX(0,H10+0.5*(D10+D11)*E11)</f>
         <v/>
       </c>
@@ -2466,7 +2552,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24">
+      <c r="A12" s="23">
         <f>Hydrogramme!A12</f>
         <v/>
       </c>
@@ -2474,7 +2560,7 @@
         <f>Hydrogramme!C12</f>
         <v/>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2482,19 +2568,19 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="24">
+      <c r="E12" s="23">
         <f>(A12-A11)*60</f>
         <v/>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="23">
         <f>0.5*(B11+B12)*E12</f>
         <v/>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="23">
         <f>F12-(H12-H11)</f>
         <v/>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="30">
         <f>MAX(0,H11+0.5*(D11+D12)*E12)</f>
         <v/>
       </c>
@@ -2504,7 +2590,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24">
+      <c r="A13" s="23">
         <f>Hydrogramme!A13</f>
         <v/>
       </c>
@@ -2512,7 +2598,7 @@
         <f>Hydrogramme!C13</f>
         <v/>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2520,19 +2606,19 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="23">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="23">
         <f>0.5*(B12+B13)*E13</f>
         <v/>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="23">
         <f>F13-(H13-H12)</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="30">
         <f>MAX(0,H12+0.5*(D12+D13)*E13)</f>
         <v/>
       </c>
@@ -2542,7 +2628,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24">
+      <c r="A14" s="23">
         <f>Hydrogramme!A14</f>
         <v/>
       </c>
@@ -2550,7 +2636,7 @@
         <f>Hydrogramme!C14</f>
         <v/>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2558,19 +2644,19 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="23">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="23">
         <f>0.5*(B13+B14)*E14</f>
         <v/>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="23">
         <f>F14-(H14-H13)</f>
         <v/>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="30">
         <f>MAX(0,H13+0.5*(D13+D14)*E14)</f>
         <v/>
       </c>
@@ -2580,7 +2666,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24">
+      <c r="A15" s="23">
         <f>Hydrogramme!A15</f>
         <v/>
       </c>
@@ -2588,7 +2674,7 @@
         <f>Hydrogramme!C15</f>
         <v/>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2596,19 +2682,19 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="23">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="23">
         <f>0.5*(B14+B15)*E15</f>
         <v/>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="23">
         <f>F15-(H15-H14)</f>
         <v/>
       </c>
-      <c r="H15" s="31">
+      <c r="H15" s="30">
         <f>MAX(0,H14+0.5*(D14+D15)*E15)</f>
         <v/>
       </c>
@@ -2618,7 +2704,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24">
+      <c r="A16" s="23">
         <f>Hydrogramme!A16</f>
         <v/>
       </c>
@@ -2626,7 +2712,7 @@
         <f>Hydrogramme!C16</f>
         <v/>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2634,19 +2720,19 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="23">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="23">
         <f>0.5*(B15+B16)*E16</f>
         <v/>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="23">
         <f>F16-(H16-H15)</f>
         <v/>
       </c>
-      <c r="H16" s="31">
+      <c r="H16" s="30">
         <f>MAX(0,H15+0.5*(D15+D16)*E16)</f>
         <v/>
       </c>
@@ -2656,7 +2742,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="24">
+      <c r="A17" s="23">
         <f>Hydrogramme!A17</f>
         <v/>
       </c>
@@ -2664,7 +2750,7 @@
         <f>Hydrogramme!C17</f>
         <v/>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2672,19 +2758,19 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="23">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="23">
         <f>0.5*(B16+B17)*E17</f>
         <v/>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="23">
         <f>F17-(H17-H16)</f>
         <v/>
       </c>
-      <c r="H17" s="31">
+      <c r="H17" s="30">
         <f>MAX(0,H16+0.5*(D16+D17)*E17)</f>
         <v/>
       </c>
@@ -2694,7 +2780,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="24">
+      <c r="A18" s="23">
         <f>Hydrogramme!A18</f>
         <v/>
       </c>
@@ -2702,7 +2788,7 @@
         <f>Hydrogramme!C18</f>
         <v/>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2710,19 +2796,19 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="23">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="23">
         <f>0.5*(B17+B18)*E18</f>
         <v/>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="23">
         <f>F18-(H18-H17)</f>
         <v/>
       </c>
-      <c r="H18" s="31">
+      <c r="H18" s="30">
         <f>MAX(0,H17+0.5*(D17+D18)*E18)</f>
         <v/>
       </c>
@@ -2732,7 +2818,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="24">
+      <c r="A19" s="23">
         <f>Hydrogramme!A19</f>
         <v/>
       </c>
@@ -2740,7 +2826,7 @@
         <f>Hydrogramme!C19</f>
         <v/>
       </c>
-      <c r="C19" s="29">
+      <c r="C19" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2748,19 +2834,19 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="23">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="23">
         <f>0.5*(B18+B19)*E19</f>
         <v/>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="23">
         <f>F19-(H19-H18)</f>
         <v/>
       </c>
-      <c r="H19" s="31">
+      <c r="H19" s="30">
         <f>MAX(0,H18+0.5*(D18+D19)*E19)</f>
         <v/>
       </c>
@@ -2770,7 +2856,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24">
+      <c r="A20" s="23">
         <f>Hydrogramme!A20</f>
         <v/>
       </c>
@@ -2778,7 +2864,7 @@
         <f>Hydrogramme!C20</f>
         <v/>
       </c>
-      <c r="C20" s="29">
+      <c r="C20" s="28">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2786,19 +2872,19 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="23">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="23">
         <f>0.5*(B19+B20)*E20</f>
         <v/>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="23">
         <f>F20-(H20-H19)</f>
         <v/>
       </c>
-      <c r="H20" s="31">
+      <c r="H20" s="30">
         <f>MAX(0,H19+0.5*(D19+D20)*E20)</f>
         <v/>
       </c>
@@ -2832,7 +2918,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Courbe de capacité Ø900 — Q = f(H) (FHWA HDS-5 inlet + outlet) — FORMULES LIVE</t>
         </is>
@@ -2872,32 +2958,32 @@
           <t>béton typ. 0.012–0.015</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="31" t="inlineStr">
         <is>
           <t>entrée</t>
         </is>
       </c>
-      <c r="F6" s="32" t="inlineStr">
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="G6" s="31" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="31" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="I6" s="32" t="inlineStr">
+      <c r="I6" s="31" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J6" s="32" t="inlineStr">
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>Ke</t>
         </is>
@@ -3013,7 +3099,7 @@
           <t>S0 = (Zin-Zout)/L</t>
         </is>
       </c>
-      <c r="B11" s="33">
+      <c r="B11" s="32">
         <f>(B9-B10)/B8</f>
         <v/>
       </c>
@@ -3044,7 +3130,7 @@
           <t>Entrée (texte exact)</t>
         </is>
       </c>
-      <c r="B13" s="34" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>square_edge</t>
         </is>
@@ -3061,7 +3147,7 @@
           <t>Q_plein Manning (réf.)</t>
         </is>
       </c>
-      <c r="B15" s="26">
+      <c r="B15" s="25">
         <f>(1/B6)*(PI()*B7^2/4)*((B7/4)^(2/3))*SQRT(B11)</f>
         <v/>
       </c>
@@ -3077,7 +3163,7 @@
           <t>K (lu)</t>
         </is>
       </c>
-      <c r="B17" s="35">
+      <c r="B17" s="34">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,2,FALSE),0.0098)</f>
         <v/>
       </c>
@@ -3088,7 +3174,7 @@
           <t>M (lu)</t>
         </is>
       </c>
-      <c r="B18" s="35">
+      <c r="B18" s="34">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,3,FALSE),2)</f>
         <v/>
       </c>
@@ -3099,7 +3185,7 @@
           <t>c (lu)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="34">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,4,FALSE),0.0398)</f>
         <v/>
       </c>
@@ -3110,7 +3196,7 @@
           <t>Y (lu)</t>
         </is>
       </c>
-      <c r="B20" s="35">
+      <c r="B20" s="34">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,5,FALSE),0.67)</f>
         <v/>
       </c>
@@ -3121,7 +3207,7 @@
           <t>Ke (lu)</t>
         </is>
       </c>
-      <c r="B21" s="35">
+      <c r="B21" s="34">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,6,FALSE),0.5)</f>
         <v/>
       </c>
@@ -3159,10 +3245,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="n">
+      <c r="A24" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="28">
         <f>$B$9+A24</f>
         <v/>
       </c>
@@ -3184,10 +3270,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="n">
+      <c r="A25" s="28" t="n">
         <v>0.05</v>
       </c>
-      <c r="B25" s="29">
+      <c r="B25" s="28">
         <f>$B$9+A25</f>
         <v/>
       </c>
@@ -3209,10 +3295,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="29" t="n">
+      <c r="A26" s="28" t="n">
         <v>0.1</v>
       </c>
-      <c r="B26" s="29">
+      <c r="B26" s="28">
         <f>$B$9+A26</f>
         <v/>
       </c>
@@ -3234,10 +3320,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="29" t="n">
+      <c r="A27" s="28" t="n">
         <v>0.15</v>
       </c>
-      <c r="B27" s="29">
+      <c r="B27" s="28">
         <f>$B$9+A27</f>
         <v/>
       </c>
@@ -3259,10 +3345,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="29" t="n">
+      <c r="A28" s="28" t="n">
         <v>0.2</v>
       </c>
-      <c r="B28" s="29">
+      <c r="B28" s="28">
         <f>$B$9+A28</f>
         <v/>
       </c>
@@ -3284,10 +3370,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="29" t="n">
+      <c r="A29" s="28" t="n">
         <v>0.25</v>
       </c>
-      <c r="B29" s="29">
+      <c r="B29" s="28">
         <f>$B$9+A29</f>
         <v/>
       </c>
@@ -3309,10 +3395,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="29" t="n">
+      <c r="A30" s="28" t="n">
         <v>0.3</v>
       </c>
-      <c r="B30" s="29">
+      <c r="B30" s="28">
         <f>$B$9+A30</f>
         <v/>
       </c>
@@ -3334,10 +3420,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="29" t="n">
+      <c r="A31" s="28" t="n">
         <v>0.35</v>
       </c>
-      <c r="B31" s="29">
+      <c r="B31" s="28">
         <f>$B$9+A31</f>
         <v/>
       </c>
@@ -3359,10 +3445,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="29" t="n">
+      <c r="A32" s="28" t="n">
         <v>0.4</v>
       </c>
-      <c r="B32" s="29">
+      <c r="B32" s="28">
         <f>$B$9+A32</f>
         <v/>
       </c>
@@ -3384,10 +3470,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="29" t="n">
+      <c r="A33" s="28" t="n">
         <v>0.45</v>
       </c>
-      <c r="B33" s="29">
+      <c r="B33" s="28">
         <f>$B$9+A33</f>
         <v/>
       </c>
@@ -3409,10 +3495,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="29" t="n">
+      <c r="A34" s="28" t="n">
         <v>0.5</v>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="28">
         <f>$B$9+A34</f>
         <v/>
       </c>
@@ -3434,10 +3520,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="29" t="n">
+      <c r="A35" s="28" t="n">
         <v>0.55</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="28">
         <f>$B$9+A35</f>
         <v/>
       </c>
@@ -3459,10 +3545,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="29" t="n">
+      <c r="A36" s="28" t="n">
         <v>0.6</v>
       </c>
-      <c r="B36" s="29">
+      <c r="B36" s="28">
         <f>$B$9+A36</f>
         <v/>
       </c>
@@ -3484,10 +3570,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="29" t="n">
+      <c r="A37" s="28" t="n">
         <v>0.65</v>
       </c>
-      <c r="B37" s="29">
+      <c r="B37" s="28">
         <f>$B$9+A37</f>
         <v/>
       </c>
@@ -3509,10 +3595,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="29" t="n">
+      <c r="A38" s="28" t="n">
         <v>0.7</v>
       </c>
-      <c r="B38" s="29">
+      <c r="B38" s="28">
         <f>$B$9+A38</f>
         <v/>
       </c>
@@ -3534,10 +3620,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="29" t="n">
+      <c r="A39" s="28" t="n">
         <v>0.75</v>
       </c>
-      <c r="B39" s="29">
+      <c r="B39" s="28">
         <f>$B$9+A39</f>
         <v/>
       </c>
@@ -3559,10 +3645,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="29" t="n">
+      <c r="A40" s="28" t="n">
         <v>0.8</v>
       </c>
-      <c r="B40" s="29">
+      <c r="B40" s="28">
         <f>$B$9+A40</f>
         <v/>
       </c>
@@ -3584,10 +3670,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="29" t="n">
+      <c r="A41" s="28" t="n">
         <v>0.85</v>
       </c>
-      <c r="B41" s="29">
+      <c r="B41" s="28">
         <f>$B$9+A41</f>
         <v/>
       </c>
@@ -3609,10 +3695,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="29" t="n">
+      <c r="A42" s="28" t="n">
         <v>0.9</v>
       </c>
-      <c r="B42" s="29">
+      <c r="B42" s="28">
         <f>$B$9+A42</f>
         <v/>
       </c>
@@ -3634,10 +3720,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="n">
+      <c r="A43" s="28" t="n">
         <v>0.95</v>
       </c>
-      <c r="B43" s="29">
+      <c r="B43" s="28">
         <f>$B$9+A43</f>
         <v/>
       </c>
@@ -3659,10 +3745,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="n">
+      <c r="A44" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="29">
+      <c r="B44" s="28">
         <f>$B$9+A44</f>
         <v/>
       </c>
@@ -3684,10 +3770,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="29" t="n">
+      <c r="A45" s="28" t="n">
         <v>1.05</v>
       </c>
-      <c r="B45" s="29">
+      <c r="B45" s="28">
         <f>$B$9+A45</f>
         <v/>
       </c>
@@ -3709,10 +3795,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="29" t="n">
+      <c r="A46" s="28" t="n">
         <v>1.1</v>
       </c>
-      <c r="B46" s="29">
+      <c r="B46" s="28">
         <f>$B$9+A46</f>
         <v/>
       </c>
@@ -3734,10 +3820,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="29" t="n">
+      <c r="A47" s="28" t="n">
         <v>1.15</v>
       </c>
-      <c r="B47" s="29">
+      <c r="B47" s="28">
         <f>$B$9+A47</f>
         <v/>
       </c>
@@ -3759,10 +3845,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="29" t="n">
+      <c r="A48" s="28" t="n">
         <v>1.2</v>
       </c>
-      <c r="B48" s="29">
+      <c r="B48" s="28">
         <f>$B$9+A48</f>
         <v/>
       </c>
@@ -3784,10 +3870,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="29" t="n">
+      <c r="A49" s="28" t="n">
         <v>1.25</v>
       </c>
-      <c r="B49" s="29">
+      <c r="B49" s="28">
         <f>$B$9+A49</f>
         <v/>
       </c>
@@ -3809,10 +3895,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="29" t="n">
+      <c r="A50" s="28" t="n">
         <v>1.3</v>
       </c>
-      <c r="B50" s="29">
+      <c r="B50" s="28">
         <f>$B$9+A50</f>
         <v/>
       </c>
@@ -3834,10 +3920,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="29" t="n">
+      <c r="A51" s="28" t="n">
         <v>1.35</v>
       </c>
-      <c r="B51" s="29">
+      <c r="B51" s="28">
         <f>$B$9+A51</f>
         <v/>
       </c>
@@ -3859,10 +3945,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="29" t="n">
+      <c r="A52" s="28" t="n">
         <v>1.4</v>
       </c>
-      <c r="B52" s="29">
+      <c r="B52" s="28">
         <f>$B$9+A52</f>
         <v/>
       </c>
@@ -3884,10 +3970,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="29" t="n">
+      <c r="A53" s="28" t="n">
         <v>1.45</v>
       </c>
-      <c r="B53" s="29">
+      <c r="B53" s="28">
         <f>$B$9+A53</f>
         <v/>
       </c>
@@ -3909,10 +3995,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="29" t="n">
+      <c r="A54" s="28" t="n">
         <v>1.5</v>
       </c>
-      <c r="B54" s="29">
+      <c r="B54" s="28">
         <f>$B$9+A54</f>
         <v/>
       </c>
@@ -3934,10 +4020,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="29" t="n">
+      <c r="A55" s="28" t="n">
         <v>1.55</v>
       </c>
-      <c r="B55" s="29">
+      <c r="B55" s="28">
         <f>$B$9+A55</f>
         <v/>
       </c>
@@ -3959,10 +4045,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="29" t="n">
+      <c r="A56" s="28" t="n">
         <v>1.6</v>
       </c>
-      <c r="B56" s="29">
+      <c r="B56" s="28">
         <f>$B$9+A56</f>
         <v/>
       </c>
@@ -3984,10 +4070,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="29" t="n">
+      <c r="A57" s="28" t="n">
         <v>1.65</v>
       </c>
-      <c r="B57" s="29">
+      <c r="B57" s="28">
         <f>$B$9+A57</f>
         <v/>
       </c>
@@ -4009,10 +4095,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="29" t="n">
+      <c r="A58" s="28" t="n">
         <v>1.7</v>
       </c>
-      <c r="B58" s="29">
+      <c r="B58" s="28">
         <f>$B$9+A58</f>
         <v/>
       </c>
@@ -4034,10 +4120,10 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="29" t="n">
+      <c r="A59" s="28" t="n">
         <v>1.75</v>
       </c>
-      <c r="B59" s="29">
+      <c r="B59" s="28">
         <f>$B$9+A59</f>
         <v/>
       </c>
@@ -4059,10 +4145,10 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="29" t="n">
+      <c r="A60" s="28" t="n">
         <v>1.8</v>
       </c>
-      <c r="B60" s="29">
+      <c r="B60" s="28">
         <f>$B$9+A60</f>
         <v/>
       </c>
@@ -4084,10 +4170,10 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="29" t="n">
+      <c r="A61" s="28" t="n">
         <v>1.85</v>
       </c>
-      <c r="B61" s="29">
+      <c r="B61" s="28">
         <f>$B$9+A61</f>
         <v/>
       </c>
@@ -4109,10 +4195,10 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="29" t="n">
+      <c r="A62" s="28" t="n">
         <v>1.9</v>
       </c>
-      <c r="B62" s="29">
+      <c r="B62" s="28">
         <f>$B$9+A62</f>
         <v/>
       </c>
@@ -4134,10 +4220,10 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="29" t="n">
+      <c r="A63" s="28" t="n">
         <v>1.95</v>
       </c>
-      <c r="B63" s="29">
+      <c r="B63" s="28">
         <f>$B$9+A63</f>
         <v/>
       </c>
@@ -4159,10 +4245,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="29" t="n">
+      <c r="A64" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="B64" s="29">
+      <c r="B64" s="28">
         <f>$B$9+A64</f>
         <v/>
       </c>
@@ -4184,10 +4270,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="29" t="n">
+      <c r="A65" s="28" t="n">
         <v>2.05</v>
       </c>
-      <c r="B65" s="29">
+      <c r="B65" s="28">
         <f>$B$9+A65</f>
         <v/>
       </c>
@@ -4209,10 +4295,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="29" t="n">
+      <c r="A66" s="28" t="n">
         <v>2.1</v>
       </c>
-      <c r="B66" s="29">
+      <c r="B66" s="28">
         <f>$B$9+A66</f>
         <v/>
       </c>
@@ -4234,10 +4320,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="29" t="n">
+      <c r="A67" s="28" t="n">
         <v>2.15</v>
       </c>
-      <c r="B67" s="29">
+      <c r="B67" s="28">
         <f>$B$9+A67</f>
         <v/>
       </c>
@@ -4259,10 +4345,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="29" t="n">
+      <c r="A68" s="28" t="n">
         <v>2.2</v>
       </c>
-      <c r="B68" s="29">
+      <c r="B68" s="28">
         <f>$B$9+A68</f>
         <v/>
       </c>
@@ -4284,10 +4370,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="29" t="n">
+      <c r="A69" s="28" t="n">
         <v>2.25</v>
       </c>
-      <c r="B69" s="29">
+      <c r="B69" s="28">
         <f>$B$9+A69</f>
         <v/>
       </c>
@@ -4309,10 +4395,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="29" t="n">
+      <c r="A70" s="28" t="n">
         <v>2.3</v>
       </c>
-      <c r="B70" s="29">
+      <c r="B70" s="28">
         <f>$B$9+A70</f>
         <v/>
       </c>
@@ -4334,10 +4420,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="29" t="n">
+      <c r="A71" s="28" t="n">
         <v>2.35</v>
       </c>
-      <c r="B71" s="29">
+      <c r="B71" s="28">
         <f>$B$9+A71</f>
         <v/>
       </c>
@@ -4359,10 +4445,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="36" t="n">
+      <c r="A72" s="35" t="n">
         <v>2.4</v>
       </c>
-      <c r="B72" s="36">
+      <c r="B72" s="35">
         <f>$B$9+A72</f>
         <v/>
       </c>
@@ -4384,10 +4470,10 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="29" t="n">
+      <c r="A73" s="28" t="n">
         <v>2.45</v>
       </c>
-      <c r="B73" s="29">
+      <c r="B73" s="28">
         <f>$B$9+A73</f>
         <v/>
       </c>
@@ -4409,10 +4495,10 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="29" t="n">
+      <c r="A74" s="28" t="n">
         <v>2.5</v>
       </c>
-      <c r="B74" s="29">
+      <c r="B74" s="28">
         <f>$B$9+A74</f>
         <v/>
       </c>
@@ -4434,10 +4520,10 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="29" t="n">
+      <c r="A75" s="28" t="n">
         <v>2.55</v>
       </c>
-      <c r="B75" s="29">
+      <c r="B75" s="28">
         <f>$B$9+A75</f>
         <v/>
       </c>
@@ -4459,10 +4545,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="29" t="n">
+      <c r="A76" s="28" t="n">
         <v>2.6</v>
       </c>
-      <c r="B76" s="29">
+      <c r="B76" s="28">
         <f>$B$9+A76</f>
         <v/>
       </c>
@@ -4484,10 +4570,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="29" t="n">
+      <c r="A77" s="28" t="n">
         <v>2.65</v>
       </c>
-      <c r="B77" s="29">
+      <c r="B77" s="28">
         <f>$B$9+A77</f>
         <v/>
       </c>
@@ -4509,10 +4595,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="29" t="n">
+      <c r="A78" s="28" t="n">
         <v>2.7</v>
       </c>
-      <c r="B78" s="29">
+      <c r="B78" s="28">
         <f>$B$9+A78</f>
         <v/>
       </c>
@@ -4534,10 +4620,10 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="29" t="n">
+      <c r="A79" s="28" t="n">
         <v>2.75</v>
       </c>
-      <c r="B79" s="29">
+      <c r="B79" s="28">
         <f>$B$9+A79</f>
         <v/>
       </c>
@@ -4559,10 +4645,10 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="29" t="n">
+      <c r="A80" s="28" t="n">
         <v>2.8</v>
       </c>
-      <c r="B80" s="29">
+      <c r="B80" s="28">
         <f>$B$9+A80</f>
         <v/>
       </c>
@@ -4584,10 +4670,10 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="29" t="n">
+      <c r="A81" s="28" t="n">
         <v>2.85</v>
       </c>
-      <c r="B81" s="29">
+      <c r="B81" s="28">
         <f>$B$9+A81</f>
         <v/>
       </c>
@@ -4609,10 +4695,10 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="29" t="n">
+      <c r="A82" s="28" t="n">
         <v>2.9</v>
       </c>
-      <c r="B82" s="29">
+      <c r="B82" s="28">
         <f>$B$9+A82</f>
         <v/>
       </c>
@@ -4634,10 +4720,10 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="29" t="n">
+      <c r="A83" s="28" t="n">
         <v>2.95</v>
       </c>
-      <c r="B83" s="29">
+      <c r="B83" s="28">
         <f>$B$9+A83</f>
         <v/>
       </c>
@@ -4659,10 +4745,10 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="29" t="n">
+      <c r="A84" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="B84" s="29">
+      <c r="B84" s="28">
         <f>$B$9+A84</f>
         <v/>
       </c>
@@ -4711,14 +4797,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Méthode B — routage avec Qout = f(H) depuis Courbe_QH_900 (FHWA)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="37" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. La courbe Courbe_QH_900 est en formules live (changer n/L/entrée/TW).</t>
         </is>
@@ -4731,7 +4817,7 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B5" s="38">
+      <c r="B5" s="37">
         <f>Parametres!B24</f>
         <v/>
       </c>
@@ -4742,7 +4828,7 @@
           <t>Q_plein réf. (m³/s)</t>
         </is>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="37">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -4753,7 +4839,7 @@
           <t>Vmax_B (m³)</t>
         </is>
       </c>
-      <c r="B7" s="28">
+      <c r="B7" s="27">
         <f>MAX(G12:G24)</f>
         <v/>
       </c>
@@ -4825,10 +4911,10 @@
         <f>MIN(B12,$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="24" t="n">
+      <c r="F12" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="31" t="n">
+      <c r="G12" s="30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4853,11 +4939,11 @@
         <f>IF(G12&lt;=0.01,MIN(0.5*(B12+B13),$B$6),D13)</f>
         <v/>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="23">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="30">
         <f>MAX(0,G12+(0.5*(B12+B13)-E13)*F13)</f>
         <v/>
       </c>
@@ -4883,11 +4969,11 @@
         <f>IF(G13&lt;=0.01,MIN(0.5*(B13+B14),$B$6),D14)</f>
         <v/>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="23">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="G14" s="31">
+      <c r="G14" s="30">
         <f>MAX(0,G13+(0.5*(B13+B14)-E14)*F14)</f>
         <v/>
       </c>
@@ -4913,11 +4999,11 @@
         <f>IF(G14&lt;=0.01,MIN(0.5*(B14+B15),$B$6),D15)</f>
         <v/>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="23">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="G15" s="31">
+      <c r="G15" s="30">
         <f>MAX(0,G14+(0.5*(B14+B15)-E15)*F15)</f>
         <v/>
       </c>
@@ -4943,11 +5029,11 @@
         <f>IF(G15&lt;=0.01,MIN(0.5*(B15+B16),$B$6),D16)</f>
         <v/>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="23">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="30">
         <f>MAX(0,G15+(0.5*(B15+B16)-E16)*F16)</f>
         <v/>
       </c>
@@ -4973,11 +5059,11 @@
         <f>IF(G16&lt;=0.01,MIN(0.5*(B16+B17),$B$6),D17)</f>
         <v/>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="23">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="G17" s="31">
+      <c r="G17" s="30">
         <f>MAX(0,G16+(0.5*(B16+B17)-E17)*F17)</f>
         <v/>
       </c>
@@ -5003,11 +5089,11 @@
         <f>IF(G17&lt;=0.01,MIN(0.5*(B17+B18),$B$6),D18)</f>
         <v/>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="23">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="G18" s="31">
+      <c r="G18" s="30">
         <f>MAX(0,G17+(0.5*(B17+B18)-E18)*F18)</f>
         <v/>
       </c>
@@ -5033,11 +5119,11 @@
         <f>IF(G18&lt;=0.01,MIN(0.5*(B18+B19),$B$6),D19)</f>
         <v/>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="23">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="G19" s="31">
+      <c r="G19" s="30">
         <f>MAX(0,G18+(0.5*(B18+B19)-E19)*F19)</f>
         <v/>
       </c>
@@ -5063,11 +5149,11 @@
         <f>IF(G19&lt;=0.01,MIN(0.5*(B19+B20),$B$6),D20)</f>
         <v/>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="23">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="30">
         <f>MAX(0,G19+(0.5*(B19+B20)-E20)*F20)</f>
         <v/>
       </c>
@@ -5093,11 +5179,11 @@
         <f>IF(G20&lt;=0.01,MIN(0.5*(B20+B21),$B$6),D21)</f>
         <v/>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="23">
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="G21" s="31">
+      <c r="G21" s="30">
         <f>MAX(0,G20+(0.5*(B20+B21)-E21)*F21)</f>
         <v/>
       </c>
@@ -5123,11 +5209,11 @@
         <f>IF(G21&lt;=0.01,MIN(0.5*(B21+B22),$B$6),D22)</f>
         <v/>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="23">
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="G22" s="31">
+      <c r="G22" s="30">
         <f>MAX(0,G21+(0.5*(B21+B22)-E22)*F22)</f>
         <v/>
       </c>
@@ -5153,11 +5239,11 @@
         <f>IF(G22&lt;=0.01,MIN(0.5*(B22+B23),$B$6),D23)</f>
         <v/>
       </c>
-      <c r="F23" s="24">
+      <c r="F23" s="23">
         <f>(A23-A22)*60</f>
         <v/>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="30">
         <f>MAX(0,G22+(0.5*(B22+B23)-E23)*F23)</f>
         <v/>
       </c>
@@ -5183,11 +5269,11 @@
         <f>IF(G23&lt;=0.01,MIN(0.5*(B23+B24),$B$6),D24)</f>
         <v/>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="23">
         <f>(A24-A23)*60</f>
         <v/>
       </c>
-      <c r="G24" s="31">
+      <c r="G24" s="30">
         <f>MAX(0,G23+(0.5*(B23+B24)-E24)*F24)</f>
         <v/>
       </c>
@@ -5206,7 +5292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5218,7 +5304,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Stage–storage du levé — V = f(WSE) → lire le niveau max</t>
         </is>
@@ -5227,7 +5313,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>PROCÉDURE (dans CE fichier): 1) Routage → Vmax sur Parametres (Calcul_A ou B). 2) Cette feuille calcule V cumulé vs NSE/WSE à partir des surfaces du levé (jaune). 3) Parametres!B30 interpolates Vmax → WSEmax. Remplacez les surfaces jaunes par vos polygones; 543 m² @ 37.28 et 1932 m² @ 39.5 sont vos mesures.</t>
+          <t>PROCÉDURE (dans CE fichier): 1) Routage → Vmax_A / Vmax_B sur Parametres (Calcul_A et Calcul_B). 2) Cette feuille calcule V cumulé vs NSE/WSE à partir des surfaces du levé (jaune). 3) Parametres!B30 = WSEmax_A (depuis Vmax_A); B36 = WSEmax_B (depuis Vmax_B). Remplacez les surfaces jaunes par vos polygones; 543 m² @ 37.28 et 1932 m² @ 39.5 sont vos mesures.</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5327,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>V_pas (m³) = (A_basse + A_haute) / 2 × (WSE_haute − WSE_basse)</t>
         </is>
@@ -5287,7 +5373,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="n">
+      <c r="A11" s="28" t="n">
         <v>34.88</v>
       </c>
       <c r="B11" s="17" t="n">
@@ -5309,21 +5395,21 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="n">
+      <c r="A12" s="28" t="n">
         <v>35.5</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>80</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="28">
         <f>A12-A11</f>
         <v/>
       </c>
-      <c r="D12" s="24">
+      <c r="D12" s="23">
         <f>0.5*(B11+B12)*C12</f>
         <v/>
       </c>
-      <c r="E12" s="31">
+      <c r="E12" s="30">
         <f>E11+D12</f>
         <v/>
       </c>
@@ -5334,21 +5420,21 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="n">
+      <c r="A13" s="28" t="n">
         <v>36</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>180</v>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="28">
         <f>A13-A12</f>
         <v/>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="23">
         <f>0.5*(B12+B13)*C13</f>
         <v/>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="30">
         <f>E12+D13</f>
         <v/>
       </c>
@@ -5359,21 +5445,21 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="n">
+      <c r="A14" s="28" t="n">
         <v>36.5</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>320</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="28">
         <f>A14-A13</f>
         <v/>
       </c>
-      <c r="D14" s="24">
+      <c r="D14" s="23">
         <f>0.5*(B13+B14)*C14</f>
         <v/>
       </c>
-      <c r="E14" s="31">
+      <c r="E14" s="30">
         <f>E13+D14</f>
         <v/>
       </c>
@@ -5384,21 +5470,21 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="n">
+      <c r="A15" s="28" t="n">
         <v>37</v>
       </c>
       <c r="B15" s="17" t="n">
         <v>480</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="28">
         <f>A15-A14</f>
         <v/>
       </c>
-      <c r="D15" s="24">
+      <c r="D15" s="23">
         <f>0.5*(B14+B15)*C15</f>
         <v/>
       </c>
-      <c r="E15" s="31">
+      <c r="E15" s="30">
         <f>E14+D15</f>
         <v/>
       </c>
@@ -5409,13 +5495,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="n">
+      <c r="A16" s="35" t="n">
         <v>37.28</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>543</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="35">
         <f>A16-A15</f>
         <v/>
       </c>
@@ -5434,21 +5520,21 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="n">
+      <c r="A17" s="28" t="n">
         <v>37.5</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>700</v>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="28">
         <f>A17-A16</f>
         <v/>
       </c>
-      <c r="D17" s="24">
+      <c r="D17" s="23">
         <f>0.5*(B16+B17)*C17</f>
         <v/>
       </c>
-      <c r="E17" s="31">
+      <c r="E17" s="30">
         <f>E16+D17</f>
         <v/>
       </c>
@@ -5459,21 +5545,21 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="n">
+      <c r="A18" s="28" t="n">
         <v>39.5</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>1932</v>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="28">
         <f>A18-A17</f>
         <v/>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="23">
         <f>0.5*(B17+B18)*C18</f>
         <v/>
       </c>
-      <c r="E18" s="31">
+      <c r="E18" s="30">
         <f>E17+D18</f>
         <v/>
       </c>
@@ -5486,7 +5572,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Vmax (depuis Calcul_A)</t>
+          <t>Vmax_A (Calcul_A)</t>
         </is>
       </c>
       <c r="B21" s="18">
@@ -5497,10 +5583,10 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>WSEmax correspondant (m)</t>
-        </is>
-      </c>
-      <c r="B22" s="21">
+          <t>WSEmax_A (m)</t>
+        </is>
+      </c>
+      <c r="B22" s="38">
         <f>Parametres!B30</f>
         <v/>
       </c>
@@ -5508,41 +5594,63 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Vmax_B (Calcul_B)</t>
+        </is>
+      </c>
+      <c r="B23" s="18">
+        <f>Parametres!B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WSEmax_B (m)</t>
+        </is>
+      </c>
+      <c r="B24" s="38">
+        <f>Parametres!B36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>V disponible à 37.28 m (m³)</t>
         </is>
       </c>
-      <c r="B23" s="40">
+      <c r="B25" s="40">
         <f>E16</f>
         <v/>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Si Vmax &gt; cette valeur → le niveau dépasse la limite patron</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Si Vmax_A ou Vmax_B &gt; cette valeur → le niveau dépasse la limite patron</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Comment lire le résultat</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="37" t="inlineStr">
-        <is>
-          <t>Exemple: si Vmax = 5609 m³ et V(37.28)≈558 m³, alors WSEmax est au-dessus de 37.28 m (la table ira vers 39.5 m ou 'Hors table'). Affinez en entrant les vraies surfaces aux cotes intermédiaires (jaune).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28"/>
+    <row r="28">
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>Exemple: si Vmax_A = 5609 m³ et V(37.28)≈558 m³, alors WSEmax_A est au-dessus de 37.28 m (la table ira vers 39.5 m ou 'Hors table'). Affinez en entrant les vraies surfaces aux cotes intermédiaires (jaune). Parametres montre WSEmax_A (B30) et WSEmax_B (B36) séparément.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A2:G4"/>
+    <mergeCell ref="A28:F30"/>
     <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A26:F28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5773,7 +5881,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8. Niveau d'eau max: Stage_Storage (surfaces levé) + Parametres!B30 = WSEmax.</t>
+          <t>8. Niveau d'eau max: Stage_Storage + Parametres!B30 (WSEmax_A) et B36 (WSEmax_B).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix fossé slope to 0.0085 and make Q_plein a live formula
S overflow default corrected from 0.085; Parametres Q_plein now
=(1/n)*A*R^(2/3)*SQRT(S0) with live A, R, S0; Qout_cap defaults to B18.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -90,12 +90,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,38 +140,39 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1752,15 +1753,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S0 = (Zamont−Zaval)/L</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="n">
-        <v>0.008489634748272452</v>
-      </c>
-      <c r="C15">
+          <t>S0 = (Zamont-Zaval)/L</t>
+        </is>
+      </c>
+      <c r="B15" s="13">
         <f>(D6-E6)/F6</f>
         <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Formule live depuis tableau géométrie Ø900</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1769,8 +1772,9 @@
           <t>A = πD²/4 (m²)</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>0.6361725123519332</v>
+      <c r="B16" s="14">
+        <f>PI()*B14^2/4</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1779,8 +1783,9 @@
           <t>R = D/4 (m)</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n">
-        <v>0.225</v>
+      <c r="B17" s="14">
+        <f>B14/4</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1789,12 +1794,13 @@
           <t>Q_plein = (1/n)·A·R^(2/3)·√S0</t>
         </is>
       </c>
-      <c r="B18" s="15" t="n">
-        <v>1.668006465155198</v>
+      <c r="B18" s="15">
+        <f>(1/B13)*B16*(B17^(2/3))*SQRT(B15)</f>
+        <v/>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>m³/s — capacité pleine section (hypothèse actuelle)</t>
+          <t>m³/s — formule live (changez n ou géométrie → Q se met à jour)</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1810,7 @@
           <t>Q utilisé avant (m³/s)</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="16" t="n">
         <v>1.77</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -1826,12 +1832,13 @@
           <t>Qout_cap_900 (m³/s)</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>1.668</v>
+      <c r="B22" s="11">
+        <f>B18</f>
+        <v/>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Par défaut = Q_plein Manning. Mettre 1.77 pour retrouver l'ancien calcul.</t>
+          <t>Par défaut = Q_plein (B18). Écraser par 1.77 si besoin (ancien calcul).</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1848,7 @@
           <t>Facteur_securite (-)</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="12" t="n">
         <v>1.2</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -1878,7 +1885,7 @@
           <t>Crest = crown Ø900 (m)</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n">
+      <c r="B27" s="12" t="n">
         <v>35.78</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -1893,7 +1900,7 @@
           <t>b fond fossé (m)</t>
         </is>
       </c>
-      <c r="B28" s="16" t="n">
+      <c r="B28" s="12" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1929,7 +1936,12 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>≈0.0085 (corrigé; pente type lit Ø900 — pas 0.085)</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -2357,7 +2369,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="43" t="inlineStr">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>
@@ -2749,7 +2761,7 @@
           <t>Qcap Ø900 (réf.)</t>
         </is>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="27">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -2796,7 +2808,7 @@
           <t>Qout (m³/s)</t>
         </is>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="28">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -2807,7 +2819,7 @@
           <t>Vmax (m³)</t>
         </is>
       </c>
-      <c r="B3" s="28">
+      <c r="B3" s="29">
         <f>MAX(H8:H20)</f>
         <v/>
       </c>
@@ -2897,7 +2909,7 @@
         <f>Hydrogramme!C8</f>
         <v/>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2914,7 +2926,7 @@
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="31" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="4">
@@ -2931,7 +2943,7 @@
         <f>Hydrogramme!C9</f>
         <v/>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2951,7 +2963,7 @@
         <f>F9-(H9-H8)</f>
         <v/>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="32">
         <f>MAX(0,H8+0.5*(D8+D9)*E9)</f>
         <v/>
       </c>
@@ -2969,7 +2981,7 @@
         <f>Hydrogramme!C10</f>
         <v/>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2989,7 +3001,7 @@
         <f>F10-(H10-H9)</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="32">
         <f>MAX(0,H9+0.5*(D9+D10)*E10)</f>
         <v/>
       </c>
@@ -3007,7 +3019,7 @@
         <f>Hydrogramme!C11</f>
         <v/>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3027,7 +3039,7 @@
         <f>F11-(H11-H10)</f>
         <v/>
       </c>
-      <c r="H11" s="31">
+      <c r="H11" s="32">
         <f>MAX(0,H10+0.5*(D10+D11)*E11)</f>
         <v/>
       </c>
@@ -3045,7 +3057,7 @@
         <f>Hydrogramme!C12</f>
         <v/>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3065,7 +3077,7 @@
         <f>F12-(H12-H11)</f>
         <v/>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="32">
         <f>MAX(0,H11+0.5*(D11+D12)*E12)</f>
         <v/>
       </c>
@@ -3083,7 +3095,7 @@
         <f>Hydrogramme!C13</f>
         <v/>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3103,7 +3115,7 @@
         <f>F13-(H13-H12)</f>
         <v/>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="32">
         <f>MAX(0,H12+0.5*(D12+D13)*E13)</f>
         <v/>
       </c>
@@ -3121,7 +3133,7 @@
         <f>Hydrogramme!C14</f>
         <v/>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3141,7 +3153,7 @@
         <f>F14-(H14-H13)</f>
         <v/>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="32">
         <f>MAX(0,H13+0.5*(D13+D14)*E14)</f>
         <v/>
       </c>
@@ -3159,7 +3171,7 @@
         <f>Hydrogramme!C15</f>
         <v/>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3179,7 +3191,7 @@
         <f>F15-(H15-H14)</f>
         <v/>
       </c>
-      <c r="H15" s="31">
+      <c r="H15" s="32">
         <f>MAX(0,H14+0.5*(D14+D15)*E15)</f>
         <v/>
       </c>
@@ -3197,7 +3209,7 @@
         <f>Hydrogramme!C16</f>
         <v/>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3217,7 +3229,7 @@
         <f>F16-(H16-H15)</f>
         <v/>
       </c>
-      <c r="H16" s="31">
+      <c r="H16" s="32">
         <f>MAX(0,H15+0.5*(D15+D16)*E16)</f>
         <v/>
       </c>
@@ -3235,7 +3247,7 @@
         <f>Hydrogramme!C17</f>
         <v/>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3255,7 +3267,7 @@
         <f>F17-(H17-H16)</f>
         <v/>
       </c>
-      <c r="H17" s="31">
+      <c r="H17" s="32">
         <f>MAX(0,H16+0.5*(D16+D17)*E17)</f>
         <v/>
       </c>
@@ -3273,7 +3285,7 @@
         <f>Hydrogramme!C18</f>
         <v/>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3293,7 +3305,7 @@
         <f>F18-(H18-H17)</f>
         <v/>
       </c>
-      <c r="H18" s="31">
+      <c r="H18" s="32">
         <f>MAX(0,H17+0.5*(D17+D18)*E18)</f>
         <v/>
       </c>
@@ -3311,7 +3323,7 @@
         <f>Hydrogramme!C19</f>
         <v/>
       </c>
-      <c r="C19" s="29">
+      <c r="C19" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3331,7 +3343,7 @@
         <f>F19-(H19-H18)</f>
         <v/>
       </c>
-      <c r="H19" s="31">
+      <c r="H19" s="32">
         <f>MAX(0,H18+0.5*(D18+D19)*E19)</f>
         <v/>
       </c>
@@ -3349,7 +3361,7 @@
         <f>Hydrogramme!C20</f>
         <v/>
       </c>
-      <c r="C20" s="29">
+      <c r="C20" s="30">
         <f>$B$2</f>
         <v/>
       </c>
@@ -3369,7 +3381,7 @@
         <f>F20-(H20-H19)</f>
         <v/>
       </c>
-      <c r="H20" s="31">
+      <c r="H20" s="32">
         <f>MAX(0,H19+0.5*(D19+D20)*E20)</f>
         <v/>
       </c>
@@ -3443,32 +3455,32 @@
           <t>béton typ. 0.012–0.015</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>entrée</t>
         </is>
       </c>
-      <c r="F6" s="32" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="G6" s="33" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="33" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="I6" s="32" t="inlineStr">
+      <c r="I6" s="33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J6" s="32" t="inlineStr">
+      <c r="J6" s="33" t="inlineStr">
         <is>
           <t>Ke</t>
         </is>
@@ -3480,7 +3492,7 @@
           <t>D (m)</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="12" t="n">
         <v>0.9</v>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -3511,7 +3523,7 @@
           <t>L (m)</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="12" t="n">
         <v>50.65</v>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -3542,7 +3554,7 @@
           <t>Radier amont Zin (m)</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="12" t="n">
         <v>34.88</v>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -3573,7 +3585,7 @@
           <t>Radier aval Zout (m)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="12" t="n">
         <v>34.45</v>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -3584,7 +3596,7 @@
           <t>S0 = (Zin-Zout)/L</t>
         </is>
       </c>
-      <c r="B11" s="33">
+      <c r="B11" s="34">
         <f>(B9-B10)/B8</f>
         <v/>
       </c>
@@ -3600,7 +3612,7 @@
           <t>TW (m au-dessus Zout)</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -3615,7 +3627,7 @@
           <t>Entrée (texte exact)</t>
         </is>
       </c>
-      <c r="B13" s="34" t="inlineStr">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>square_edge</t>
         </is>
@@ -3648,7 +3660,7 @@
           <t>K (lu)</t>
         </is>
       </c>
-      <c r="B17" s="35">
+      <c r="B17" s="36">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,2,FALSE),0.0098)</f>
         <v/>
       </c>
@@ -3659,7 +3671,7 @@
           <t>M (lu)</t>
         </is>
       </c>
-      <c r="B18" s="35">
+      <c r="B18" s="36">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,3,FALSE),2)</f>
         <v/>
       </c>
@@ -3670,7 +3682,7 @@
           <t>c (lu)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="36">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,4,FALSE),0.0398)</f>
         <v/>
       </c>
@@ -3681,7 +3693,7 @@
           <t>Y (lu)</t>
         </is>
       </c>
-      <c r="B20" s="35">
+      <c r="B20" s="36">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,5,FALSE),0.67)</f>
         <v/>
       </c>
@@ -3692,7 +3704,7 @@
           <t>Ke (lu)</t>
         </is>
       </c>
-      <c r="B21" s="35">
+      <c r="B21" s="36">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,6,FALSE),0.5)</f>
         <v/>
       </c>
@@ -3730,10 +3742,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="n">
+      <c r="A24" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="30">
         <f>$B$9+A24</f>
         <v/>
       </c>
@@ -3755,10 +3767,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="n">
+      <c r="A25" s="30" t="n">
         <v>0.05</v>
       </c>
-      <c r="B25" s="29">
+      <c r="B25" s="30">
         <f>$B$9+A25</f>
         <v/>
       </c>
@@ -3780,10 +3792,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="29" t="n">
+      <c r="A26" s="30" t="n">
         <v>0.1</v>
       </c>
-      <c r="B26" s="29">
+      <c r="B26" s="30">
         <f>$B$9+A26</f>
         <v/>
       </c>
@@ -3805,10 +3817,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="29" t="n">
+      <c r="A27" s="30" t="n">
         <v>0.15</v>
       </c>
-      <c r="B27" s="29">
+      <c r="B27" s="30">
         <f>$B$9+A27</f>
         <v/>
       </c>
@@ -3830,10 +3842,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="29" t="n">
+      <c r="A28" s="30" t="n">
         <v>0.2</v>
       </c>
-      <c r="B28" s="29">
+      <c r="B28" s="30">
         <f>$B$9+A28</f>
         <v/>
       </c>
@@ -3855,10 +3867,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="29" t="n">
+      <c r="A29" s="30" t="n">
         <v>0.25</v>
       </c>
-      <c r="B29" s="29">
+      <c r="B29" s="30">
         <f>$B$9+A29</f>
         <v/>
       </c>
@@ -3880,10 +3892,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="29" t="n">
+      <c r="A30" s="30" t="n">
         <v>0.3</v>
       </c>
-      <c r="B30" s="29">
+      <c r="B30" s="30">
         <f>$B$9+A30</f>
         <v/>
       </c>
@@ -3905,10 +3917,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="29" t="n">
+      <c r="A31" s="30" t="n">
         <v>0.35</v>
       </c>
-      <c r="B31" s="29">
+      <c r="B31" s="30">
         <f>$B$9+A31</f>
         <v/>
       </c>
@@ -3930,10 +3942,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="29" t="n">
+      <c r="A32" s="30" t="n">
         <v>0.4</v>
       </c>
-      <c r="B32" s="29">
+      <c r="B32" s="30">
         <f>$B$9+A32</f>
         <v/>
       </c>
@@ -3955,10 +3967,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="29" t="n">
+      <c r="A33" s="30" t="n">
         <v>0.45</v>
       </c>
-      <c r="B33" s="29">
+      <c r="B33" s="30">
         <f>$B$9+A33</f>
         <v/>
       </c>
@@ -3980,10 +3992,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="29" t="n">
+      <c r="A34" s="30" t="n">
         <v>0.5</v>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="30">
         <f>$B$9+A34</f>
         <v/>
       </c>
@@ -4005,10 +4017,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="29" t="n">
+      <c r="A35" s="30" t="n">
         <v>0.55</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="30">
         <f>$B$9+A35</f>
         <v/>
       </c>
@@ -4030,10 +4042,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="29" t="n">
+      <c r="A36" s="30" t="n">
         <v>0.6</v>
       </c>
-      <c r="B36" s="29">
+      <c r="B36" s="30">
         <f>$B$9+A36</f>
         <v/>
       </c>
@@ -4055,10 +4067,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="29" t="n">
+      <c r="A37" s="30" t="n">
         <v>0.65</v>
       </c>
-      <c r="B37" s="29">
+      <c r="B37" s="30">
         <f>$B$9+A37</f>
         <v/>
       </c>
@@ -4080,10 +4092,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="29" t="n">
+      <c r="A38" s="30" t="n">
         <v>0.7</v>
       </c>
-      <c r="B38" s="29">
+      <c r="B38" s="30">
         <f>$B$9+A38</f>
         <v/>
       </c>
@@ -4105,10 +4117,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="29" t="n">
+      <c r="A39" s="30" t="n">
         <v>0.75</v>
       </c>
-      <c r="B39" s="29">
+      <c r="B39" s="30">
         <f>$B$9+A39</f>
         <v/>
       </c>
@@ -4130,10 +4142,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="29" t="n">
+      <c r="A40" s="30" t="n">
         <v>0.8</v>
       </c>
-      <c r="B40" s="29">
+      <c r="B40" s="30">
         <f>$B$9+A40</f>
         <v/>
       </c>
@@ -4155,10 +4167,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="29" t="n">
+      <c r="A41" s="30" t="n">
         <v>0.85</v>
       </c>
-      <c r="B41" s="29">
+      <c r="B41" s="30">
         <f>$B$9+A41</f>
         <v/>
       </c>
@@ -4180,10 +4192,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="29" t="n">
+      <c r="A42" s="30" t="n">
         <v>0.9</v>
       </c>
-      <c r="B42" s="29">
+      <c r="B42" s="30">
         <f>$B$9+A42</f>
         <v/>
       </c>
@@ -4205,10 +4217,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="n">
+      <c r="A43" s="30" t="n">
         <v>0.95</v>
       </c>
-      <c r="B43" s="29">
+      <c r="B43" s="30">
         <f>$B$9+A43</f>
         <v/>
       </c>
@@ -4230,10 +4242,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="n">
+      <c r="A44" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="29">
+      <c r="B44" s="30">
         <f>$B$9+A44</f>
         <v/>
       </c>
@@ -4255,10 +4267,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="29" t="n">
+      <c r="A45" s="30" t="n">
         <v>1.05</v>
       </c>
-      <c r="B45" s="29">
+      <c r="B45" s="30">
         <f>$B$9+A45</f>
         <v/>
       </c>
@@ -4280,10 +4292,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="29" t="n">
+      <c r="A46" s="30" t="n">
         <v>1.1</v>
       </c>
-      <c r="B46" s="29">
+      <c r="B46" s="30">
         <f>$B$9+A46</f>
         <v/>
       </c>
@@ -4305,10 +4317,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="29" t="n">
+      <c r="A47" s="30" t="n">
         <v>1.15</v>
       </c>
-      <c r="B47" s="29">
+      <c r="B47" s="30">
         <f>$B$9+A47</f>
         <v/>
       </c>
@@ -4330,10 +4342,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="29" t="n">
+      <c r="A48" s="30" t="n">
         <v>1.2</v>
       </c>
-      <c r="B48" s="29">
+      <c r="B48" s="30">
         <f>$B$9+A48</f>
         <v/>
       </c>
@@ -4355,10 +4367,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="29" t="n">
+      <c r="A49" s="30" t="n">
         <v>1.25</v>
       </c>
-      <c r="B49" s="29">
+      <c r="B49" s="30">
         <f>$B$9+A49</f>
         <v/>
       </c>
@@ -4380,10 +4392,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="29" t="n">
+      <c r="A50" s="30" t="n">
         <v>1.3</v>
       </c>
-      <c r="B50" s="29">
+      <c r="B50" s="30">
         <f>$B$9+A50</f>
         <v/>
       </c>
@@ -4405,10 +4417,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="29" t="n">
+      <c r="A51" s="30" t="n">
         <v>1.35</v>
       </c>
-      <c r="B51" s="29">
+      <c r="B51" s="30">
         <f>$B$9+A51</f>
         <v/>
       </c>
@@ -4430,10 +4442,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="29" t="n">
+      <c r="A52" s="30" t="n">
         <v>1.4</v>
       </c>
-      <c r="B52" s="29">
+      <c r="B52" s="30">
         <f>$B$9+A52</f>
         <v/>
       </c>
@@ -4455,10 +4467,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="29" t="n">
+      <c r="A53" s="30" t="n">
         <v>1.45</v>
       </c>
-      <c r="B53" s="29">
+      <c r="B53" s="30">
         <f>$B$9+A53</f>
         <v/>
       </c>
@@ -4480,10 +4492,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="29" t="n">
+      <c r="A54" s="30" t="n">
         <v>1.5</v>
       </c>
-      <c r="B54" s="29">
+      <c r="B54" s="30">
         <f>$B$9+A54</f>
         <v/>
       </c>
@@ -4505,10 +4517,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="29" t="n">
+      <c r="A55" s="30" t="n">
         <v>1.55</v>
       </c>
-      <c r="B55" s="29">
+      <c r="B55" s="30">
         <f>$B$9+A55</f>
         <v/>
       </c>
@@ -4530,10 +4542,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="29" t="n">
+      <c r="A56" s="30" t="n">
         <v>1.6</v>
       </c>
-      <c r="B56" s="29">
+      <c r="B56" s="30">
         <f>$B$9+A56</f>
         <v/>
       </c>
@@ -4555,10 +4567,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="29" t="n">
+      <c r="A57" s="30" t="n">
         <v>1.65</v>
       </c>
-      <c r="B57" s="29">
+      <c r="B57" s="30">
         <f>$B$9+A57</f>
         <v/>
       </c>
@@ -4580,10 +4592,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="29" t="n">
+      <c r="A58" s="30" t="n">
         <v>1.7</v>
       </c>
-      <c r="B58" s="29">
+      <c r="B58" s="30">
         <f>$B$9+A58</f>
         <v/>
       </c>
@@ -4605,10 +4617,10 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="29" t="n">
+      <c r="A59" s="30" t="n">
         <v>1.75</v>
       </c>
-      <c r="B59" s="29">
+      <c r="B59" s="30">
         <f>$B$9+A59</f>
         <v/>
       </c>
@@ -4630,10 +4642,10 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="29" t="n">
+      <c r="A60" s="30" t="n">
         <v>1.8</v>
       </c>
-      <c r="B60" s="29">
+      <c r="B60" s="30">
         <f>$B$9+A60</f>
         <v/>
       </c>
@@ -4655,10 +4667,10 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="29" t="n">
+      <c r="A61" s="30" t="n">
         <v>1.85</v>
       </c>
-      <c r="B61" s="29">
+      <c r="B61" s="30">
         <f>$B$9+A61</f>
         <v/>
       </c>
@@ -4680,10 +4692,10 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="29" t="n">
+      <c r="A62" s="30" t="n">
         <v>1.9</v>
       </c>
-      <c r="B62" s="29">
+      <c r="B62" s="30">
         <f>$B$9+A62</f>
         <v/>
       </c>
@@ -4705,10 +4717,10 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="29" t="n">
+      <c r="A63" s="30" t="n">
         <v>1.95</v>
       </c>
-      <c r="B63" s="29">
+      <c r="B63" s="30">
         <f>$B$9+A63</f>
         <v/>
       </c>
@@ -4730,10 +4742,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="29" t="n">
+      <c r="A64" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="B64" s="29">
+      <c r="B64" s="30">
         <f>$B$9+A64</f>
         <v/>
       </c>
@@ -4755,10 +4767,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="29" t="n">
+      <c r="A65" s="30" t="n">
         <v>2.05</v>
       </c>
-      <c r="B65" s="29">
+      <c r="B65" s="30">
         <f>$B$9+A65</f>
         <v/>
       </c>
@@ -4780,10 +4792,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="29" t="n">
+      <c r="A66" s="30" t="n">
         <v>2.1</v>
       </c>
-      <c r="B66" s="29">
+      <c r="B66" s="30">
         <f>$B$9+A66</f>
         <v/>
       </c>
@@ -4805,10 +4817,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="29" t="n">
+      <c r="A67" s="30" t="n">
         <v>2.15</v>
       </c>
-      <c r="B67" s="29">
+      <c r="B67" s="30">
         <f>$B$9+A67</f>
         <v/>
       </c>
@@ -4830,10 +4842,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="29" t="n">
+      <c r="A68" s="30" t="n">
         <v>2.2</v>
       </c>
-      <c r="B68" s="29">
+      <c r="B68" s="30">
         <f>$B$9+A68</f>
         <v/>
       </c>
@@ -4855,10 +4867,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="29" t="n">
+      <c r="A69" s="30" t="n">
         <v>2.25</v>
       </c>
-      <c r="B69" s="29">
+      <c r="B69" s="30">
         <f>$B$9+A69</f>
         <v/>
       </c>
@@ -4880,10 +4892,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="29" t="n">
+      <c r="A70" s="30" t="n">
         <v>2.3</v>
       </c>
-      <c r="B70" s="29">
+      <c r="B70" s="30">
         <f>$B$9+A70</f>
         <v/>
       </c>
@@ -4905,10 +4917,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="29" t="n">
+      <c r="A71" s="30" t="n">
         <v>2.35</v>
       </c>
-      <c r="B71" s="29">
+      <c r="B71" s="30">
         <f>$B$9+A71</f>
         <v/>
       </c>
@@ -4930,10 +4942,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="36" t="n">
+      <c r="A72" s="37" t="n">
         <v>2.4</v>
       </c>
-      <c r="B72" s="36">
+      <c r="B72" s="37">
         <f>$B$9+A72</f>
         <v/>
       </c>
@@ -4955,10 +4967,10 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="29" t="n">
+      <c r="A73" s="30" t="n">
         <v>2.45</v>
       </c>
-      <c r="B73" s="29">
+      <c r="B73" s="30">
         <f>$B$9+A73</f>
         <v/>
       </c>
@@ -4980,10 +4992,10 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="29" t="n">
+      <c r="A74" s="30" t="n">
         <v>2.5</v>
       </c>
-      <c r="B74" s="29">
+      <c r="B74" s="30">
         <f>$B$9+A74</f>
         <v/>
       </c>
@@ -5005,10 +5017,10 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="29" t="n">
+      <c r="A75" s="30" t="n">
         <v>2.55</v>
       </c>
-      <c r="B75" s="29">
+      <c r="B75" s="30">
         <f>$B$9+A75</f>
         <v/>
       </c>
@@ -5030,10 +5042,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="29" t="n">
+      <c r="A76" s="30" t="n">
         <v>2.6</v>
       </c>
-      <c r="B76" s="29">
+      <c r="B76" s="30">
         <f>$B$9+A76</f>
         <v/>
       </c>
@@ -5055,10 +5067,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="29" t="n">
+      <c r="A77" s="30" t="n">
         <v>2.65</v>
       </c>
-      <c r="B77" s="29">
+      <c r="B77" s="30">
         <f>$B$9+A77</f>
         <v/>
       </c>
@@ -5080,10 +5092,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="29" t="n">
+      <c r="A78" s="30" t="n">
         <v>2.7</v>
       </c>
-      <c r="B78" s="29">
+      <c r="B78" s="30">
         <f>$B$9+A78</f>
         <v/>
       </c>
@@ -5105,10 +5117,10 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="29" t="n">
+      <c r="A79" s="30" t="n">
         <v>2.75</v>
       </c>
-      <c r="B79" s="29">
+      <c r="B79" s="30">
         <f>$B$9+A79</f>
         <v/>
       </c>
@@ -5130,10 +5142,10 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="29" t="n">
+      <c r="A80" s="30" t="n">
         <v>2.8</v>
       </c>
-      <c r="B80" s="29">
+      <c r="B80" s="30">
         <f>$B$9+A80</f>
         <v/>
       </c>
@@ -5155,10 +5167,10 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="29" t="n">
+      <c r="A81" s="30" t="n">
         <v>2.85</v>
       </c>
-      <c r="B81" s="29">
+      <c r="B81" s="30">
         <f>$B$9+A81</f>
         <v/>
       </c>
@@ -5180,10 +5192,10 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="29" t="n">
+      <c r="A82" s="30" t="n">
         <v>2.9</v>
       </c>
-      <c r="B82" s="29">
+      <c r="B82" s="30">
         <f>$B$9+A82</f>
         <v/>
       </c>
@@ -5205,10 +5217,10 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="29" t="n">
+      <c r="A83" s="30" t="n">
         <v>2.95</v>
       </c>
-      <c r="B83" s="29">
+      <c r="B83" s="30">
         <f>$B$9+A83</f>
         <v/>
       </c>
@@ -5230,10 +5242,10 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="29" t="n">
+      <c r="A84" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="B84" s="29">
+      <c r="B84" s="30">
         <f>$B$9+A84</f>
         <v/>
       </c>
@@ -5289,7 +5301,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="37" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. La courbe Courbe_QH_900 est en formules live (changer n/L/entrée/TW).</t>
         </is>
@@ -5302,7 +5314,7 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B5" s="38">
+      <c r="B5" s="39">
         <f>Parametres!B24</f>
         <v/>
       </c>
@@ -5313,7 +5325,7 @@
           <t>Q_plein réf. (m³/s)</t>
         </is>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="39">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -5324,7 +5336,7 @@
           <t>Vmax_B (m³)</t>
         </is>
       </c>
-      <c r="B7" s="28">
+      <c r="B7" s="29">
         <f>MAX(G12:G24)</f>
         <v/>
       </c>
@@ -5399,7 +5411,7 @@
       <c r="F12" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="31" t="n">
+      <c r="G12" s="32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5428,7 +5440,7 @@
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="32">
         <f>MAX(0,G12+(0.5*(B12+B13)-E13)*F13)</f>
         <v/>
       </c>
@@ -5458,7 +5470,7 @@
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="G14" s="31">
+      <c r="G14" s="32">
         <f>MAX(0,G13+(0.5*(B13+B14)-E14)*F14)</f>
         <v/>
       </c>
@@ -5488,7 +5500,7 @@
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="G15" s="31">
+      <c r="G15" s="32">
         <f>MAX(0,G14+(0.5*(B14+B15)-E15)*F15)</f>
         <v/>
       </c>
@@ -5518,7 +5530,7 @@
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="32">
         <f>MAX(0,G15+(0.5*(B15+B16)-E16)*F16)</f>
         <v/>
       </c>
@@ -5548,7 +5560,7 @@
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="G17" s="31">
+      <c r="G17" s="32">
         <f>MAX(0,G16+(0.5*(B16+B17)-E17)*F17)</f>
         <v/>
       </c>
@@ -5578,7 +5590,7 @@
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="G18" s="31">
+      <c r="G18" s="32">
         <f>MAX(0,G17+(0.5*(B17+B18)-E18)*F18)</f>
         <v/>
       </c>
@@ -5608,7 +5620,7 @@
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="G19" s="31">
+      <c r="G19" s="32">
         <f>MAX(0,G18+(0.5*(B18+B19)-E19)*F19)</f>
         <v/>
       </c>
@@ -5638,7 +5650,7 @@
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="32">
         <f>MAX(0,G19+(0.5*(B19+B20)-E20)*F20)</f>
         <v/>
       </c>
@@ -5668,7 +5680,7 @@
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="G21" s="31">
+      <c r="G21" s="32">
         <f>MAX(0,G20+(0.5*(B20+B21)-E21)*F21)</f>
         <v/>
       </c>
@@ -5698,7 +5710,7 @@
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="G22" s="31">
+      <c r="G22" s="32">
         <f>MAX(0,G21+(0.5*(B21+B22)-E22)*F22)</f>
         <v/>
       </c>
@@ -5728,7 +5740,7 @@
         <f>(A23-A22)*60</f>
         <v/>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="32">
         <f>MAX(0,G22+(0.5*(B22+B23)-E23)*F23)</f>
         <v/>
       </c>
@@ -5758,7 +5770,7 @@
         <f>(A24-A23)*60</f>
         <v/>
       </c>
-      <c r="G24" s="31">
+      <c r="G24" s="32">
         <f>MAX(0,G23+(0.5*(B23+B24)-E24)*F24)</f>
         <v/>
       </c>
@@ -5821,7 +5833,7 @@
           <t>Crest (m)</t>
         </is>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="12">
         <f>Parametres!B27</f>
         <v/>
       </c>
@@ -5832,7 +5844,7 @@
           <t>b (m)</t>
         </is>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="12">
         <f>Parametres!B28</f>
         <v/>
       </c>
@@ -5887,7 +5899,7 @@
           <t>Zin Ø900 (m)</t>
         </is>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="12">
         <f>34.88</f>
         <v/>
       </c>
@@ -5950,14 +5962,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="n">
+      <c r="A15" s="30" t="n">
         <v>34.88</v>
       </c>
-      <c r="B15" s="29">
+      <c r="B15" s="30">
         <f>A15-$B$12</f>
         <v/>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="30">
         <f>MAX(0,A15-$B$6)</f>
         <v/>
       </c>
@@ -5973,7 +5985,7 @@
         <f>IF(A15&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A15&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A15,Stage_Storage!$A$11:$A$18,1))+(A15-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A15,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A15,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A15,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A15,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A15,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G15" s="31">
+      <c r="G15" s="32">
         <f>E15+F15</f>
         <v/>
       </c>
@@ -5995,14 +6007,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="n">
+      <c r="A16" s="30" t="n">
         <v>34.93</v>
       </c>
-      <c r="B16" s="29">
+      <c r="B16" s="30">
         <f>A16-$B$12</f>
         <v/>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="30">
         <f>MAX(0,A16-$B$6)</f>
         <v/>
       </c>
@@ -6018,7 +6030,7 @@
         <f>IF(A16&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A16&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A16,Stage_Storage!$A$11:$A$18,1))+(A16-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A16,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A16,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A16,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A16,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A16,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="32">
         <f>E16+F16</f>
         <v/>
       </c>
@@ -6040,14 +6052,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="n">
+      <c r="A17" s="30" t="n">
         <v>34.98</v>
       </c>
-      <c r="B17" s="29">
+      <c r="B17" s="30">
         <f>A17-$B$12</f>
         <v/>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="30">
         <f>MAX(0,A17-$B$6)</f>
         <v/>
       </c>
@@ -6063,7 +6075,7 @@
         <f>IF(A17&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A17&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A17,Stage_Storage!$A$11:$A$18,1))+(A17-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A17,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A17,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A17,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A17,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A17,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G17" s="31">
+      <c r="G17" s="32">
         <f>E17+F17</f>
         <v/>
       </c>
@@ -6085,14 +6097,14 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="n">
+      <c r="A18" s="30" t="n">
         <v>35.03</v>
       </c>
-      <c r="B18" s="29">
+      <c r="B18" s="30">
         <f>A18-$B$12</f>
         <v/>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="30">
         <f>MAX(0,A18-$B$6)</f>
         <v/>
       </c>
@@ -6108,7 +6120,7 @@
         <f>IF(A18&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A18&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A18,Stage_Storage!$A$11:$A$18,1))+(A18-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A18,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A18,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A18,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A18,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A18,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G18" s="31">
+      <c r="G18" s="32">
         <f>E18+F18</f>
         <v/>
       </c>
@@ -6130,14 +6142,14 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="n">
+      <c r="A19" s="30" t="n">
         <v>35.08</v>
       </c>
-      <c r="B19" s="29">
+      <c r="B19" s="30">
         <f>A19-$B$12</f>
         <v/>
       </c>
-      <c r="C19" s="29">
+      <c r="C19" s="30">
         <f>MAX(0,A19-$B$6)</f>
         <v/>
       </c>
@@ -6153,7 +6165,7 @@
         <f>IF(A19&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A19&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A19,Stage_Storage!$A$11:$A$18,1))+(A19-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A19,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A19,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A19,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A19,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A19,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G19" s="31">
+      <c r="G19" s="32">
         <f>E19+F19</f>
         <v/>
       </c>
@@ -6175,14 +6187,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="n">
+      <c r="A20" s="30" t="n">
         <v>35.13</v>
       </c>
-      <c r="B20" s="29">
+      <c r="B20" s="30">
         <f>A20-$B$12</f>
         <v/>
       </c>
-      <c r="C20" s="29">
+      <c r="C20" s="30">
         <f>MAX(0,A20-$B$6)</f>
         <v/>
       </c>
@@ -6198,7 +6210,7 @@
         <f>IF(A20&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A20&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A20,Stage_Storage!$A$11:$A$18,1))+(A20-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A20,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A20,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A20,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A20,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A20,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="32">
         <f>E20+F20</f>
         <v/>
       </c>
@@ -6220,14 +6232,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="n">
+      <c r="A21" s="30" t="n">
         <v>35.18</v>
       </c>
-      <c r="B21" s="29">
+      <c r="B21" s="30">
         <f>A21-$B$12</f>
         <v/>
       </c>
-      <c r="C21" s="29">
+      <c r="C21" s="30">
         <f>MAX(0,A21-$B$6)</f>
         <v/>
       </c>
@@ -6243,7 +6255,7 @@
         <f>IF(A21&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A21&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A21,Stage_Storage!$A$11:$A$18,1))+(A21-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A21,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A21,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A21,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A21,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A21,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G21" s="31">
+      <c r="G21" s="32">
         <f>E21+F21</f>
         <v/>
       </c>
@@ -6265,14 +6277,14 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="n">
+      <c r="A22" s="30" t="n">
         <v>35.23</v>
       </c>
-      <c r="B22" s="29">
+      <c r="B22" s="30">
         <f>A22-$B$12</f>
         <v/>
       </c>
-      <c r="C22" s="29">
+      <c r="C22" s="30">
         <f>MAX(0,A22-$B$6)</f>
         <v/>
       </c>
@@ -6288,7 +6300,7 @@
         <f>IF(A22&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A22&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A22,Stage_Storage!$A$11:$A$18,1))+(A22-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A22,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A22,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A22,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A22,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A22,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G22" s="31">
+      <c r="G22" s="32">
         <f>E22+F22</f>
         <v/>
       </c>
@@ -6310,14 +6322,14 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="n">
+      <c r="A23" s="30" t="n">
         <v>35.28</v>
       </c>
-      <c r="B23" s="29">
+      <c r="B23" s="30">
         <f>A23-$B$12</f>
         <v/>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="30">
         <f>MAX(0,A23-$B$6)</f>
         <v/>
       </c>
@@ -6333,7 +6345,7 @@
         <f>IF(A23&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A23&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A23,Stage_Storage!$A$11:$A$18,1))+(A23-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A23,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A23,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A23,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A23,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A23,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="32">
         <f>E23+F23</f>
         <v/>
       </c>
@@ -6355,14 +6367,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="n">
+      <c r="A24" s="30" t="n">
         <v>35.33</v>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="30">
         <f>A24-$B$12</f>
         <v/>
       </c>
-      <c r="C24" s="29">
+      <c r="C24" s="30">
         <f>MAX(0,A24-$B$6)</f>
         <v/>
       </c>
@@ -6378,7 +6390,7 @@
         <f>IF(A24&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A24&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A24,Stage_Storage!$A$11:$A$18,1))+(A24-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A24,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A24,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A24,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A24,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A24,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G24" s="31">
+      <c r="G24" s="32">
         <f>E24+F24</f>
         <v/>
       </c>
@@ -6400,14 +6412,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="n">
+      <c r="A25" s="30" t="n">
         <v>35.38</v>
       </c>
-      <c r="B25" s="29">
+      <c r="B25" s="30">
         <f>A25-$B$12</f>
         <v/>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="30">
         <f>MAX(0,A25-$B$6)</f>
         <v/>
       </c>
@@ -6423,7 +6435,7 @@
         <f>IF(A25&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A25&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A25,Stage_Storage!$A$11:$A$18,1))+(A25-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A25,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A25,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A25,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A25,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A25,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G25" s="31">
+      <c r="G25" s="32">
         <f>E25+F25</f>
         <v/>
       </c>
@@ -6445,14 +6457,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="29" t="n">
+      <c r="A26" s="30" t="n">
         <v>35.43</v>
       </c>
-      <c r="B26" s="29">
+      <c r="B26" s="30">
         <f>A26-$B$12</f>
         <v/>
       </c>
-      <c r="C26" s="29">
+      <c r="C26" s="30">
         <f>MAX(0,A26-$B$6)</f>
         <v/>
       </c>
@@ -6468,7 +6480,7 @@
         <f>IF(A26&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A26&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A26,Stage_Storage!$A$11:$A$18,1))+(A26-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A26,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A26,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A26,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A26,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A26,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G26" s="31">
+      <c r="G26" s="32">
         <f>E26+F26</f>
         <v/>
       </c>
@@ -6490,14 +6502,14 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="29" t="n">
+      <c r="A27" s="30" t="n">
         <v>35.48</v>
       </c>
-      <c r="B27" s="29">
+      <c r="B27" s="30">
         <f>A27-$B$12</f>
         <v/>
       </c>
-      <c r="C27" s="29">
+      <c r="C27" s="30">
         <f>MAX(0,A27-$B$6)</f>
         <v/>
       </c>
@@ -6513,7 +6525,7 @@
         <f>IF(A27&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A27&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A27,Stage_Storage!$A$11:$A$18,1))+(A27-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A27,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A27,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A27,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A27,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A27,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G27" s="31">
+      <c r="G27" s="32">
         <f>E27+F27</f>
         <v/>
       </c>
@@ -6535,14 +6547,14 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="29" t="n">
+      <c r="A28" s="30" t="n">
         <v>35.53</v>
       </c>
-      <c r="B28" s="29">
+      <c r="B28" s="30">
         <f>A28-$B$12</f>
         <v/>
       </c>
-      <c r="C28" s="29">
+      <c r="C28" s="30">
         <f>MAX(0,A28-$B$6)</f>
         <v/>
       </c>
@@ -6558,7 +6570,7 @@
         <f>IF(A28&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A28&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A28,Stage_Storage!$A$11:$A$18,1))+(A28-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A28,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A28,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A28,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A28,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A28,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G28" s="31">
+      <c r="G28" s="32">
         <f>E28+F28</f>
         <v/>
       </c>
@@ -6580,14 +6592,14 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="29" t="n">
+      <c r="A29" s="30" t="n">
         <v>35.58</v>
       </c>
-      <c r="B29" s="29">
+      <c r="B29" s="30">
         <f>A29-$B$12</f>
         <v/>
       </c>
-      <c r="C29" s="29">
+      <c r="C29" s="30">
         <f>MAX(0,A29-$B$6)</f>
         <v/>
       </c>
@@ -6603,7 +6615,7 @@
         <f>IF(A29&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A29&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A29,Stage_Storage!$A$11:$A$18,1))+(A29-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A29,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A29,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A29,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A29,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A29,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G29" s="31">
+      <c r="G29" s="32">
         <f>E29+F29</f>
         <v/>
       </c>
@@ -6625,14 +6637,14 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="29" t="n">
+      <c r="A30" s="30" t="n">
         <v>35.63</v>
       </c>
-      <c r="B30" s="29">
+      <c r="B30" s="30">
         <f>A30-$B$12</f>
         <v/>
       </c>
-      <c r="C30" s="29">
+      <c r="C30" s="30">
         <f>MAX(0,A30-$B$6)</f>
         <v/>
       </c>
@@ -6648,7 +6660,7 @@
         <f>IF(A30&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A30&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A30,Stage_Storage!$A$11:$A$18,1))+(A30-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A30,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A30,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A30,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A30,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A30,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G30" s="31">
+      <c r="G30" s="32">
         <f>E30+F30</f>
         <v/>
       </c>
@@ -6670,14 +6682,14 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="29" t="n">
+      <c r="A31" s="30" t="n">
         <v>35.68</v>
       </c>
-      <c r="B31" s="29">
+      <c r="B31" s="30">
         <f>A31-$B$12</f>
         <v/>
       </c>
-      <c r="C31" s="29">
+      <c r="C31" s="30">
         <f>MAX(0,A31-$B$6)</f>
         <v/>
       </c>
@@ -6693,7 +6705,7 @@
         <f>IF(A31&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A31&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A31,Stage_Storage!$A$11:$A$18,1))+(A31-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A31,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A31,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A31,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A31,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A31,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G31" s="31">
+      <c r="G31" s="32">
         <f>E31+F31</f>
         <v/>
       </c>
@@ -6715,14 +6727,14 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="29" t="n">
+      <c r="A32" s="30" t="n">
         <v>35.73</v>
       </c>
-      <c r="B32" s="29">
+      <c r="B32" s="30">
         <f>A32-$B$12</f>
         <v/>
       </c>
-      <c r="C32" s="29">
+      <c r="C32" s="30">
         <f>MAX(0,A32-$B$6)</f>
         <v/>
       </c>
@@ -6738,7 +6750,7 @@
         <f>IF(A32&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A32&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A32,Stage_Storage!$A$11:$A$18,1))+(A32-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A32,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A32,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A32,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A32,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A32,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G32" s="31">
+      <c r="G32" s="32">
         <f>E32+F32</f>
         <v/>
       </c>
@@ -6760,14 +6772,14 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="36" t="n">
+      <c r="A33" s="37" t="n">
         <v>35.78</v>
       </c>
-      <c r="B33" s="36">
+      <c r="B33" s="37">
         <f>A33-$B$12</f>
         <v/>
       </c>
-      <c r="C33" s="36">
+      <c r="C33" s="37">
         <f>MAX(0,A33-$B$6)</f>
         <v/>
       </c>
@@ -6775,15 +6787,15 @@
         <f>IF(C33&lt;=0,0,($B$7+$B$9*C33)*C33)</f>
         <v/>
       </c>
-      <c r="E33" s="39">
+      <c r="E33" s="40">
         <f>D33*$B$11</f>
         <v/>
       </c>
-      <c r="F33" s="39">
+      <c r="F33" s="40">
         <f>IF(A33&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A33&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A33,Stage_Storage!$A$11:$A$18,1))+(A33-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A33,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A33,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A33,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A33,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A33,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G33" s="31">
+      <c r="G33" s="32">
         <f>E33+F33</f>
         <v/>
       </c>
@@ -6805,14 +6817,14 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="29" t="n">
+      <c r="A34" s="30" t="n">
         <v>35.83</v>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="30">
         <f>A34-$B$12</f>
         <v/>
       </c>
-      <c r="C34" s="29">
+      <c r="C34" s="30">
         <f>MAX(0,A34-$B$6)</f>
         <v/>
       </c>
@@ -6828,7 +6840,7 @@
         <f>IF(A34&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A34&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A34,Stage_Storage!$A$11:$A$18,1))+(A34-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A34,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A34,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A34,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A34,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A34,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G34" s="31">
+      <c r="G34" s="32">
         <f>E34+F34</f>
         <v/>
       </c>
@@ -6850,14 +6862,14 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="29" t="n">
+      <c r="A35" s="30" t="n">
         <v>35.88</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="30">
         <f>A35-$B$12</f>
         <v/>
       </c>
-      <c r="C35" s="29">
+      <c r="C35" s="30">
         <f>MAX(0,A35-$B$6)</f>
         <v/>
       </c>
@@ -6873,7 +6885,7 @@
         <f>IF(A35&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A35&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A35,Stage_Storage!$A$11:$A$18,1))+(A35-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A35,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A35,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A35,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A35,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A35,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G35" s="31">
+      <c r="G35" s="32">
         <f>E35+F35</f>
         <v/>
       </c>
@@ -6895,14 +6907,14 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="29" t="n">
+      <c r="A36" s="30" t="n">
         <v>35.93</v>
       </c>
-      <c r="B36" s="29">
+      <c r="B36" s="30">
         <f>A36-$B$12</f>
         <v/>
       </c>
-      <c r="C36" s="29">
+      <c r="C36" s="30">
         <f>MAX(0,A36-$B$6)</f>
         <v/>
       </c>
@@ -6918,7 +6930,7 @@
         <f>IF(A36&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A36&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A36,Stage_Storage!$A$11:$A$18,1))+(A36-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A36,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A36,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A36,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A36,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A36,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G36" s="31">
+      <c r="G36" s="32">
         <f>E36+F36</f>
         <v/>
       </c>
@@ -6940,14 +6952,14 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="29" t="n">
+      <c r="A37" s="30" t="n">
         <v>35.98</v>
       </c>
-      <c r="B37" s="29">
+      <c r="B37" s="30">
         <f>A37-$B$12</f>
         <v/>
       </c>
-      <c r="C37" s="29">
+      <c r="C37" s="30">
         <f>MAX(0,A37-$B$6)</f>
         <v/>
       </c>
@@ -6963,7 +6975,7 @@
         <f>IF(A37&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A37&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A37,Stage_Storage!$A$11:$A$18,1))+(A37-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A37,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A37,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A37,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A37,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A37,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G37" s="31">
+      <c r="G37" s="32">
         <f>E37+F37</f>
         <v/>
       </c>
@@ -6985,14 +6997,14 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="29" t="n">
+      <c r="A38" s="30" t="n">
         <v>36.03</v>
       </c>
-      <c r="B38" s="29">
+      <c r="B38" s="30">
         <f>A38-$B$12</f>
         <v/>
       </c>
-      <c r="C38" s="29">
+      <c r="C38" s="30">
         <f>MAX(0,A38-$B$6)</f>
         <v/>
       </c>
@@ -7008,7 +7020,7 @@
         <f>IF(A38&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A38&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A38,Stage_Storage!$A$11:$A$18,1))+(A38-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A38,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A38,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A38,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A38,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A38,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G38" s="31">
+      <c r="G38" s="32">
         <f>E38+F38</f>
         <v/>
       </c>
@@ -7030,14 +7042,14 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="29" t="n">
+      <c r="A39" s="30" t="n">
         <v>36.08</v>
       </c>
-      <c r="B39" s="29">
+      <c r="B39" s="30">
         <f>A39-$B$12</f>
         <v/>
       </c>
-      <c r="C39" s="29">
+      <c r="C39" s="30">
         <f>MAX(0,A39-$B$6)</f>
         <v/>
       </c>
@@ -7053,7 +7065,7 @@
         <f>IF(A39&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A39&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A39,Stage_Storage!$A$11:$A$18,1))+(A39-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A39,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A39,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A39,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A39,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A39,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G39" s="31">
+      <c r="G39" s="32">
         <f>E39+F39</f>
         <v/>
       </c>
@@ -7075,14 +7087,14 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="29" t="n">
+      <c r="A40" s="30" t="n">
         <v>36.13</v>
       </c>
-      <c r="B40" s="29">
+      <c r="B40" s="30">
         <f>A40-$B$12</f>
         <v/>
       </c>
-      <c r="C40" s="29">
+      <c r="C40" s="30">
         <f>MAX(0,A40-$B$6)</f>
         <v/>
       </c>
@@ -7098,7 +7110,7 @@
         <f>IF(A40&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A40&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A40,Stage_Storage!$A$11:$A$18,1))+(A40-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A40,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A40,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A40,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A40,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A40,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G40" s="31">
+      <c r="G40" s="32">
         <f>E40+F40</f>
         <v/>
       </c>
@@ -7120,14 +7132,14 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="29" t="n">
+      <c r="A41" s="30" t="n">
         <v>36.18</v>
       </c>
-      <c r="B41" s="29">
+      <c r="B41" s="30">
         <f>A41-$B$12</f>
         <v/>
       </c>
-      <c r="C41" s="29">
+      <c r="C41" s="30">
         <f>MAX(0,A41-$B$6)</f>
         <v/>
       </c>
@@ -7143,7 +7155,7 @@
         <f>IF(A41&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A41&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A41,Stage_Storage!$A$11:$A$18,1))+(A41-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A41,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A41,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A41,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A41,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A41,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G41" s="31">
+      <c r="G41" s="32">
         <f>E41+F41</f>
         <v/>
       </c>
@@ -7165,14 +7177,14 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="29" t="n">
+      <c r="A42" s="30" t="n">
         <v>36.23</v>
       </c>
-      <c r="B42" s="29">
+      <c r="B42" s="30">
         <f>A42-$B$12</f>
         <v/>
       </c>
-      <c r="C42" s="29">
+      <c r="C42" s="30">
         <f>MAX(0,A42-$B$6)</f>
         <v/>
       </c>
@@ -7188,7 +7200,7 @@
         <f>IF(A42&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A42&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A42,Stage_Storage!$A$11:$A$18,1))+(A42-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A42,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A42,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A42,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A42,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A42,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G42" s="31">
+      <c r="G42" s="32">
         <f>E42+F42</f>
         <v/>
       </c>
@@ -7210,14 +7222,14 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="n">
+      <c r="A43" s="30" t="n">
         <v>36.28</v>
       </c>
-      <c r="B43" s="29">
+      <c r="B43" s="30">
         <f>A43-$B$12</f>
         <v/>
       </c>
-      <c r="C43" s="29">
+      <c r="C43" s="30">
         <f>MAX(0,A43-$B$6)</f>
         <v/>
       </c>
@@ -7233,7 +7245,7 @@
         <f>IF(A43&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A43&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A43,Stage_Storage!$A$11:$A$18,1))+(A43-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A43,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A43,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A43,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A43,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A43,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G43" s="31">
+      <c r="G43" s="32">
         <f>E43+F43</f>
         <v/>
       </c>
@@ -7255,14 +7267,14 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="n">
+      <c r="A44" s="30" t="n">
         <v>36.33</v>
       </c>
-      <c r="B44" s="29">
+      <c r="B44" s="30">
         <f>A44-$B$12</f>
         <v/>
       </c>
-      <c r="C44" s="29">
+      <c r="C44" s="30">
         <f>MAX(0,A44-$B$6)</f>
         <v/>
       </c>
@@ -7278,7 +7290,7 @@
         <f>IF(A44&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A44&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A44,Stage_Storage!$A$11:$A$18,1))+(A44-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A44,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A44,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A44,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A44,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A44,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G44" s="31">
+      <c r="G44" s="32">
         <f>E44+F44</f>
         <v/>
       </c>
@@ -7300,14 +7312,14 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="29" t="n">
+      <c r="A45" s="30" t="n">
         <v>36.38</v>
       </c>
-      <c r="B45" s="29">
+      <c r="B45" s="30">
         <f>A45-$B$12</f>
         <v/>
       </c>
-      <c r="C45" s="29">
+      <c r="C45" s="30">
         <f>MAX(0,A45-$B$6)</f>
         <v/>
       </c>
@@ -7323,7 +7335,7 @@
         <f>IF(A45&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A45&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A45,Stage_Storage!$A$11:$A$18,1))+(A45-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A45,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A45,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A45,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A45,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A45,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G45" s="31">
+      <c r="G45" s="32">
         <f>E45+F45</f>
         <v/>
       </c>
@@ -7345,14 +7357,14 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="29" t="n">
+      <c r="A46" s="30" t="n">
         <v>36.43</v>
       </c>
-      <c r="B46" s="29">
+      <c r="B46" s="30">
         <f>A46-$B$12</f>
         <v/>
       </c>
-      <c r="C46" s="29">
+      <c r="C46" s="30">
         <f>MAX(0,A46-$B$6)</f>
         <v/>
       </c>
@@ -7368,7 +7380,7 @@
         <f>IF(A46&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A46&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A46,Stage_Storage!$A$11:$A$18,1))+(A46-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A46,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A46,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A46,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A46,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A46,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G46" s="31">
+      <c r="G46" s="32">
         <f>E46+F46</f>
         <v/>
       </c>
@@ -7390,14 +7402,14 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="29" t="n">
+      <c r="A47" s="30" t="n">
         <v>36.48</v>
       </c>
-      <c r="B47" s="29">
+      <c r="B47" s="30">
         <f>A47-$B$12</f>
         <v/>
       </c>
-      <c r="C47" s="29">
+      <c r="C47" s="30">
         <f>MAX(0,A47-$B$6)</f>
         <v/>
       </c>
@@ -7413,7 +7425,7 @@
         <f>IF(A47&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A47&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A47,Stage_Storage!$A$11:$A$18,1))+(A47-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A47,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A47,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A47,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A47,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A47,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G47" s="31">
+      <c r="G47" s="32">
         <f>E47+F47</f>
         <v/>
       </c>
@@ -7435,14 +7447,14 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="29" t="n">
+      <c r="A48" s="30" t="n">
         <v>36.53</v>
       </c>
-      <c r="B48" s="29">
+      <c r="B48" s="30">
         <f>A48-$B$12</f>
         <v/>
       </c>
-      <c r="C48" s="29">
+      <c r="C48" s="30">
         <f>MAX(0,A48-$B$6)</f>
         <v/>
       </c>
@@ -7458,7 +7470,7 @@
         <f>IF(A48&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A48&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A48,Stage_Storage!$A$11:$A$18,1))+(A48-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A48,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A48,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A48,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A48,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A48,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G48" s="31">
+      <c r="G48" s="32">
         <f>E48+F48</f>
         <v/>
       </c>
@@ -7480,14 +7492,14 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="29" t="n">
+      <c r="A49" s="30" t="n">
         <v>36.58</v>
       </c>
-      <c r="B49" s="29">
+      <c r="B49" s="30">
         <f>A49-$B$12</f>
         <v/>
       </c>
-      <c r="C49" s="29">
+      <c r="C49" s="30">
         <f>MAX(0,A49-$B$6)</f>
         <v/>
       </c>
@@ -7503,7 +7515,7 @@
         <f>IF(A49&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A49&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A49,Stage_Storage!$A$11:$A$18,1))+(A49-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A49,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A49,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A49,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A49,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A49,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G49" s="31">
+      <c r="G49" s="32">
         <f>E49+F49</f>
         <v/>
       </c>
@@ -7525,14 +7537,14 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="29" t="n">
+      <c r="A50" s="30" t="n">
         <v>36.63</v>
       </c>
-      <c r="B50" s="29">
+      <c r="B50" s="30">
         <f>A50-$B$12</f>
         <v/>
       </c>
-      <c r="C50" s="29">
+      <c r="C50" s="30">
         <f>MAX(0,A50-$B$6)</f>
         <v/>
       </c>
@@ -7548,7 +7560,7 @@
         <f>IF(A50&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A50&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A50,Stage_Storage!$A$11:$A$18,1))+(A50-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A50,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A50,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A50,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A50,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A50,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G50" s="31">
+      <c r="G50" s="32">
         <f>E50+F50</f>
         <v/>
       </c>
@@ -7570,14 +7582,14 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="29" t="n">
+      <c r="A51" s="30" t="n">
         <v>36.68</v>
       </c>
-      <c r="B51" s="29">
+      <c r="B51" s="30">
         <f>A51-$B$12</f>
         <v/>
       </c>
-      <c r="C51" s="29">
+      <c r="C51" s="30">
         <f>MAX(0,A51-$B$6)</f>
         <v/>
       </c>
@@ -7593,7 +7605,7 @@
         <f>IF(A51&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A51&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A51,Stage_Storage!$A$11:$A$18,1))+(A51-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A51,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A51,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A51,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A51,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A51,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G51" s="31">
+      <c r="G51" s="32">
         <f>E51+F51</f>
         <v/>
       </c>
@@ -7615,14 +7627,14 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="29" t="n">
+      <c r="A52" s="30" t="n">
         <v>36.73</v>
       </c>
-      <c r="B52" s="29">
+      <c r="B52" s="30">
         <f>A52-$B$12</f>
         <v/>
       </c>
-      <c r="C52" s="29">
+      <c r="C52" s="30">
         <f>MAX(0,A52-$B$6)</f>
         <v/>
       </c>
@@ -7638,7 +7650,7 @@
         <f>IF(A52&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A52&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A52,Stage_Storage!$A$11:$A$18,1))+(A52-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A52,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A52,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A52,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A52,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A52,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G52" s="31">
+      <c r="G52" s="32">
         <f>E52+F52</f>
         <v/>
       </c>
@@ -7660,14 +7672,14 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="29" t="n">
+      <c r="A53" s="30" t="n">
         <v>36.78</v>
       </c>
-      <c r="B53" s="29">
+      <c r="B53" s="30">
         <f>A53-$B$12</f>
         <v/>
       </c>
-      <c r="C53" s="29">
+      <c r="C53" s="30">
         <f>MAX(0,A53-$B$6)</f>
         <v/>
       </c>
@@ -7683,7 +7695,7 @@
         <f>IF(A53&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A53&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A53,Stage_Storage!$A$11:$A$18,1))+(A53-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A53,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A53,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A53,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A53,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A53,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G53" s="31">
+      <c r="G53" s="32">
         <f>E53+F53</f>
         <v/>
       </c>
@@ -7705,14 +7717,14 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="29" t="n">
+      <c r="A54" s="30" t="n">
         <v>36.83</v>
       </c>
-      <c r="B54" s="29">
+      <c r="B54" s="30">
         <f>A54-$B$12</f>
         <v/>
       </c>
-      <c r="C54" s="29">
+      <c r="C54" s="30">
         <f>MAX(0,A54-$B$6)</f>
         <v/>
       </c>
@@ -7728,7 +7740,7 @@
         <f>IF(A54&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A54&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A54,Stage_Storage!$A$11:$A$18,1))+(A54-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A54,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A54,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A54,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A54,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A54,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G54" s="31">
+      <c r="G54" s="32">
         <f>E54+F54</f>
         <v/>
       </c>
@@ -7750,14 +7762,14 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="29" t="n">
+      <c r="A55" s="30" t="n">
         <v>36.88</v>
       </c>
-      <c r="B55" s="29">
+      <c r="B55" s="30">
         <f>A55-$B$12</f>
         <v/>
       </c>
-      <c r="C55" s="29">
+      <c r="C55" s="30">
         <f>MAX(0,A55-$B$6)</f>
         <v/>
       </c>
@@ -7773,7 +7785,7 @@
         <f>IF(A55&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A55&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A55,Stage_Storage!$A$11:$A$18,1))+(A55-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A55,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A55,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A55,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A55,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A55,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G55" s="31">
+      <c r="G55" s="32">
         <f>E55+F55</f>
         <v/>
       </c>
@@ -7795,14 +7807,14 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="29" t="n">
+      <c r="A56" s="30" t="n">
         <v>36.93</v>
       </c>
-      <c r="B56" s="29">
+      <c r="B56" s="30">
         <f>A56-$B$12</f>
         <v/>
       </c>
-      <c r="C56" s="29">
+      <c r="C56" s="30">
         <f>MAX(0,A56-$B$6)</f>
         <v/>
       </c>
@@ -7818,7 +7830,7 @@
         <f>IF(A56&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A56&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A56,Stage_Storage!$A$11:$A$18,1))+(A56-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A56,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A56,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A56,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A56,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A56,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G56" s="31">
+      <c r="G56" s="32">
         <f>E56+F56</f>
         <v/>
       </c>
@@ -7840,14 +7852,14 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="29" t="n">
+      <c r="A57" s="30" t="n">
         <v>36.98</v>
       </c>
-      <c r="B57" s="29">
+      <c r="B57" s="30">
         <f>A57-$B$12</f>
         <v/>
       </c>
-      <c r="C57" s="29">
+      <c r="C57" s="30">
         <f>MAX(0,A57-$B$6)</f>
         <v/>
       </c>
@@ -7863,7 +7875,7 @@
         <f>IF(A57&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A57&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A57,Stage_Storage!$A$11:$A$18,1))+(A57-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A57,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A57,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A57,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A57,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A57,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G57" s="31">
+      <c r="G57" s="32">
         <f>E57+F57</f>
         <v/>
       </c>
@@ -7885,14 +7897,14 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="29" t="n">
+      <c r="A58" s="30" t="n">
         <v>37.03</v>
       </c>
-      <c r="B58" s="29">
+      <c r="B58" s="30">
         <f>A58-$B$12</f>
         <v/>
       </c>
-      <c r="C58" s="29">
+      <c r="C58" s="30">
         <f>MAX(0,A58-$B$6)</f>
         <v/>
       </c>
@@ -7908,7 +7920,7 @@
         <f>IF(A58&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A58&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A58,Stage_Storage!$A$11:$A$18,1))+(A58-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A58,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A58,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A58,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A58,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A58,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G58" s="31">
+      <c r="G58" s="32">
         <f>E58+F58</f>
         <v/>
       </c>
@@ -7930,14 +7942,14 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="29" t="n">
+      <c r="A59" s="30" t="n">
         <v>37.08</v>
       </c>
-      <c r="B59" s="29">
+      <c r="B59" s="30">
         <f>A59-$B$12</f>
         <v/>
       </c>
-      <c r="C59" s="29">
+      <c r="C59" s="30">
         <f>MAX(0,A59-$B$6)</f>
         <v/>
       </c>
@@ -7953,7 +7965,7 @@
         <f>IF(A59&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A59&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A59,Stage_Storage!$A$11:$A$18,1))+(A59-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A59,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A59,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A59,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A59,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A59,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G59" s="31">
+      <c r="G59" s="32">
         <f>E59+F59</f>
         <v/>
       </c>
@@ -7975,14 +7987,14 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="29" t="n">
+      <c r="A60" s="30" t="n">
         <v>37.13</v>
       </c>
-      <c r="B60" s="29">
+      <c r="B60" s="30">
         <f>A60-$B$12</f>
         <v/>
       </c>
-      <c r="C60" s="29">
+      <c r="C60" s="30">
         <f>MAX(0,A60-$B$6)</f>
         <v/>
       </c>
@@ -7998,7 +8010,7 @@
         <f>IF(A60&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A60&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1))+(A60-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G60" s="31">
+      <c r="G60" s="32">
         <f>E60+F60</f>
         <v/>
       </c>
@@ -8020,14 +8032,14 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="29" t="n">
+      <c r="A61" s="30" t="n">
         <v>37.18</v>
       </c>
-      <c r="B61" s="29">
+      <c r="B61" s="30">
         <f>A61-$B$12</f>
         <v/>
       </c>
-      <c r="C61" s="29">
+      <c r="C61" s="30">
         <f>MAX(0,A61-$B$6)</f>
         <v/>
       </c>
@@ -8043,7 +8055,7 @@
         <f>IF(A61&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A61&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1))+(A61-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G61" s="31">
+      <c r="G61" s="32">
         <f>E61+F61</f>
         <v/>
       </c>
@@ -8065,14 +8077,14 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="29" t="n">
+      <c r="A62" s="30" t="n">
         <v>37.23</v>
       </c>
-      <c r="B62" s="29">
+      <c r="B62" s="30">
         <f>A62-$B$12</f>
         <v/>
       </c>
-      <c r="C62" s="29">
+      <c r="C62" s="30">
         <f>MAX(0,A62-$B$6)</f>
         <v/>
       </c>
@@ -8088,7 +8100,7 @@
         <f>IF(A62&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A62&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1))+(A62-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G62" s="31">
+      <c r="G62" s="32">
         <f>E62+F62</f>
         <v/>
       </c>
@@ -8110,14 +8122,14 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="29" t="n">
+      <c r="A63" s="30" t="n">
         <v>37.28</v>
       </c>
-      <c r="B63" s="29">
+      <c r="B63" s="30">
         <f>A63-$B$12</f>
         <v/>
       </c>
-      <c r="C63" s="29">
+      <c r="C63" s="30">
         <f>MAX(0,A63-$B$6)</f>
         <v/>
       </c>
@@ -8133,7 +8145,7 @@
         <f>IF(A63&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A63&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1))+(A63-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G63" s="31">
+      <c r="G63" s="32">
         <f>E63+F63</f>
         <v/>
       </c>
@@ -8155,14 +8167,14 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="29" t="n">
+      <c r="A64" s="30" t="n">
         <v>37.33</v>
       </c>
-      <c r="B64" s="29">
+      <c r="B64" s="30">
         <f>A64-$B$12</f>
         <v/>
       </c>
-      <c r="C64" s="29">
+      <c r="C64" s="30">
         <f>MAX(0,A64-$B$6)</f>
         <v/>
       </c>
@@ -8178,7 +8190,7 @@
         <f>IF(A64&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A64&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1))+(A64-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G64" s="31">
+      <c r="G64" s="32">
         <f>E64+F64</f>
         <v/>
       </c>
@@ -8200,14 +8212,14 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="29" t="n">
+      <c r="A65" s="30" t="n">
         <v>37.38</v>
       </c>
-      <c r="B65" s="29">
+      <c r="B65" s="30">
         <f>A65-$B$12</f>
         <v/>
       </c>
-      <c r="C65" s="29">
+      <c r="C65" s="30">
         <f>MAX(0,A65-$B$6)</f>
         <v/>
       </c>
@@ -8223,7 +8235,7 @@
         <f>IF(A65&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A65&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1))+(A65-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A65,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G65" s="31">
+      <c r="G65" s="32">
         <f>E65+F65</f>
         <v/>
       </c>
@@ -8245,14 +8257,14 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="29" t="n">
+      <c r="A66" s="30" t="n">
         <v>37.43</v>
       </c>
-      <c r="B66" s="29">
+      <c r="B66" s="30">
         <f>A66-$B$12</f>
         <v/>
       </c>
-      <c r="C66" s="29">
+      <c r="C66" s="30">
         <f>MAX(0,A66-$B$6)</f>
         <v/>
       </c>
@@ -8268,7 +8280,7 @@
         <f>IF(A66&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A66&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1))+(A66-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A66,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G66" s="31">
+      <c r="G66" s="32">
         <f>E66+F66</f>
         <v/>
       </c>
@@ -8290,14 +8302,14 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="29" t="n">
+      <c r="A67" s="30" t="n">
         <v>37.48</v>
       </c>
-      <c r="B67" s="29">
+      <c r="B67" s="30">
         <f>A67-$B$12</f>
         <v/>
       </c>
-      <c r="C67" s="29">
+      <c r="C67" s="30">
         <f>MAX(0,A67-$B$6)</f>
         <v/>
       </c>
@@ -8313,7 +8325,7 @@
         <f>IF(A67&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A67&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A67,Stage_Storage!$A$11:$A$18,1))+(A67-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A67,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A67,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A67,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A67,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A67,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G67" s="31">
+      <c r="G67" s="32">
         <f>E67+F67</f>
         <v/>
       </c>
@@ -8335,14 +8347,14 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="29" t="n">
+      <c r="A68" s="30" t="n">
         <v>37.53</v>
       </c>
-      <c r="B68" s="29">
+      <c r="B68" s="30">
         <f>A68-$B$12</f>
         <v/>
       </c>
-      <c r="C68" s="29">
+      <c r="C68" s="30">
         <f>MAX(0,A68-$B$6)</f>
         <v/>
       </c>
@@ -8358,7 +8370,7 @@
         <f>IF(A68&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A68&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A68,Stage_Storage!$A$11:$A$18,1))+(A68-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A68,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A68,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A68,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A68,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A68,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G68" s="31">
+      <c r="G68" s="32">
         <f>E68+F68</f>
         <v/>
       </c>
@@ -8380,14 +8392,14 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="29" t="n">
+      <c r="A69" s="30" t="n">
         <v>37.58</v>
       </c>
-      <c r="B69" s="29">
+      <c r="B69" s="30">
         <f>A69-$B$12</f>
         <v/>
       </c>
-      <c r="C69" s="29">
+      <c r="C69" s="30">
         <f>MAX(0,A69-$B$6)</f>
         <v/>
       </c>
@@ -8403,7 +8415,7 @@
         <f>IF(A69&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A69&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A69,Stage_Storage!$A$11:$A$18,1))+(A69-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A69,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A69,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A69,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A69,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A69,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G69" s="31">
+      <c r="G69" s="32">
         <f>E69+F69</f>
         <v/>
       </c>
@@ -8425,14 +8437,14 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="29" t="n">
+      <c r="A70" s="30" t="n">
         <v>37.63</v>
       </c>
-      <c r="B70" s="29">
+      <c r="B70" s="30">
         <f>A70-$B$12</f>
         <v/>
       </c>
-      <c r="C70" s="29">
+      <c r="C70" s="30">
         <f>MAX(0,A70-$B$6)</f>
         <v/>
       </c>
@@ -8448,7 +8460,7 @@
         <f>IF(A70&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A70&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A70,Stage_Storage!$A$11:$A$18,1))+(A70-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A70,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A70,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A70,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A70,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A70,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G70" s="31">
+      <c r="G70" s="32">
         <f>E70+F70</f>
         <v/>
       </c>
@@ -8470,14 +8482,14 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="29" t="n">
+      <c r="A71" s="30" t="n">
         <v>37.68</v>
       </c>
-      <c r="B71" s="29">
+      <c r="B71" s="30">
         <f>A71-$B$12</f>
         <v/>
       </c>
-      <c r="C71" s="29">
+      <c r="C71" s="30">
         <f>MAX(0,A71-$B$6)</f>
         <v/>
       </c>
@@ -8493,7 +8505,7 @@
         <f>IF(A71&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A71&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A71,Stage_Storage!$A$11:$A$18,1))+(A71-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A71,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A71,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A71,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A71,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A71,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G71" s="31">
+      <c r="G71" s="32">
         <f>E71+F71</f>
         <v/>
       </c>
@@ -8515,14 +8527,14 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="29" t="n">
+      <c r="A72" s="30" t="n">
         <v>37.73</v>
       </c>
-      <c r="B72" s="29">
+      <c r="B72" s="30">
         <f>A72-$B$12</f>
         <v/>
       </c>
-      <c r="C72" s="29">
+      <c r="C72" s="30">
         <f>MAX(0,A72-$B$6)</f>
         <v/>
       </c>
@@ -8538,7 +8550,7 @@
         <f>IF(A72&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A72&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A72,Stage_Storage!$A$11:$A$18,1))+(A72-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A72,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A72,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A72,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A72,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A72,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G72" s="31">
+      <c r="G72" s="32">
         <f>E72+F72</f>
         <v/>
       </c>
@@ -8560,14 +8572,14 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="29" t="n">
+      <c r="A73" s="30" t="n">
         <v>37.78</v>
       </c>
-      <c r="B73" s="29">
+      <c r="B73" s="30">
         <f>A73-$B$12</f>
         <v/>
       </c>
-      <c r="C73" s="29">
+      <c r="C73" s="30">
         <f>MAX(0,A73-$B$6)</f>
         <v/>
       </c>
@@ -8583,7 +8595,7 @@
         <f>IF(A73&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A73&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A73,Stage_Storage!$A$11:$A$18,1))+(A73-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A73,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A73,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A73,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A73,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A73,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G73" s="31">
+      <c r="G73" s="32">
         <f>E73+F73</f>
         <v/>
       </c>
@@ -8605,14 +8617,14 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="29" t="n">
+      <c r="A74" s="30" t="n">
         <v>37.83</v>
       </c>
-      <c r="B74" s="29">
+      <c r="B74" s="30">
         <f>A74-$B$12</f>
         <v/>
       </c>
-      <c r="C74" s="29">
+      <c r="C74" s="30">
         <f>MAX(0,A74-$B$6)</f>
         <v/>
       </c>
@@ -8628,7 +8640,7 @@
         <f>IF(A74&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A74&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A74,Stage_Storage!$A$11:$A$18,1))+(A74-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A74,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A74,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A74,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A74,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A74,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G74" s="31">
+      <c r="G74" s="32">
         <f>E74+F74</f>
         <v/>
       </c>
@@ -8650,14 +8662,14 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="29" t="n">
+      <c r="A75" s="30" t="n">
         <v>37.88</v>
       </c>
-      <c r="B75" s="29">
+      <c r="B75" s="30">
         <f>A75-$B$12</f>
         <v/>
       </c>
-      <c r="C75" s="29">
+      <c r="C75" s="30">
         <f>MAX(0,A75-$B$6)</f>
         <v/>
       </c>
@@ -8673,7 +8685,7 @@
         <f>IF(A75&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A75&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A75,Stage_Storage!$A$11:$A$18,1))+(A75-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A75,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A75,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A75,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A75,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A75,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G75" s="31">
+      <c r="G75" s="32">
         <f>E75+F75</f>
         <v/>
       </c>
@@ -8695,14 +8707,14 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="29" t="n">
+      <c r="A76" s="30" t="n">
         <v>37.93</v>
       </c>
-      <c r="B76" s="29">
+      <c r="B76" s="30">
         <f>A76-$B$12</f>
         <v/>
       </c>
-      <c r="C76" s="29">
+      <c r="C76" s="30">
         <f>MAX(0,A76-$B$6)</f>
         <v/>
       </c>
@@ -8718,7 +8730,7 @@
         <f>IF(A76&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A76&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A76,Stage_Storage!$A$11:$A$18,1))+(A76-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A76,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A76,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A76,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A76,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A76,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G76" s="31">
+      <c r="G76" s="32">
         <f>E76+F76</f>
         <v/>
       </c>
@@ -8740,14 +8752,14 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="29" t="n">
+      <c r="A77" s="30" t="n">
         <v>37.98</v>
       </c>
-      <c r="B77" s="29">
+      <c r="B77" s="30">
         <f>A77-$B$12</f>
         <v/>
       </c>
-      <c r="C77" s="29">
+      <c r="C77" s="30">
         <f>MAX(0,A77-$B$6)</f>
         <v/>
       </c>
@@ -8763,7 +8775,7 @@
         <f>IF(A77&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A77&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A77,Stage_Storage!$A$11:$A$18,1))+(A77-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A77,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A77,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A77,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A77,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A77,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G77" s="31">
+      <c r="G77" s="32">
         <f>E77+F77</f>
         <v/>
       </c>
@@ -8785,14 +8797,14 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="29" t="n">
+      <c r="A78" s="30" t="n">
         <v>38.03</v>
       </c>
-      <c r="B78" s="29">
+      <c r="B78" s="30">
         <f>A78-$B$12</f>
         <v/>
       </c>
-      <c r="C78" s="29">
+      <c r="C78" s="30">
         <f>MAX(0,A78-$B$6)</f>
         <v/>
       </c>
@@ -8808,7 +8820,7 @@
         <f>IF(A78&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A78&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A78,Stage_Storage!$A$11:$A$18,1))+(A78-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A78,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A78,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A78,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A78,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A78,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G78" s="31">
+      <c r="G78" s="32">
         <f>E78+F78</f>
         <v/>
       </c>
@@ -8830,14 +8842,14 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="29" t="n">
+      <c r="A79" s="30" t="n">
         <v>38.08</v>
       </c>
-      <c r="B79" s="29">
+      <c r="B79" s="30">
         <f>A79-$B$12</f>
         <v/>
       </c>
-      <c r="C79" s="29">
+      <c r="C79" s="30">
         <f>MAX(0,A79-$B$6)</f>
         <v/>
       </c>
@@ -8853,7 +8865,7 @@
         <f>IF(A79&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A79&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A79,Stage_Storage!$A$11:$A$18,1))+(A79-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A79,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A79,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A79,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A79,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A79,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G79" s="31">
+      <c r="G79" s="32">
         <f>E79+F79</f>
         <v/>
       </c>
@@ -8875,14 +8887,14 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="29" t="n">
+      <c r="A80" s="30" t="n">
         <v>38.13</v>
       </c>
-      <c r="B80" s="29">
+      <c r="B80" s="30">
         <f>A80-$B$12</f>
         <v/>
       </c>
-      <c r="C80" s="29">
+      <c r="C80" s="30">
         <f>MAX(0,A80-$B$6)</f>
         <v/>
       </c>
@@ -8898,7 +8910,7 @@
         <f>IF(A80&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A80&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A80,Stage_Storage!$A$11:$A$18,1))+(A80-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A80,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A80,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A80,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A80,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A80,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G80" s="31">
+      <c r="G80" s="32">
         <f>E80+F80</f>
         <v/>
       </c>
@@ -8920,14 +8932,14 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="29" t="n">
+      <c r="A81" s="30" t="n">
         <v>38.18</v>
       </c>
-      <c r="B81" s="29">
+      <c r="B81" s="30">
         <f>A81-$B$12</f>
         <v/>
       </c>
-      <c r="C81" s="29">
+      <c r="C81" s="30">
         <f>MAX(0,A81-$B$6)</f>
         <v/>
       </c>
@@ -8943,7 +8955,7 @@
         <f>IF(A81&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A81&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A81,Stage_Storage!$A$11:$A$18,1))+(A81-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A81,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A81,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A81,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A81,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A81,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G81" s="31">
+      <c r="G81" s="32">
         <f>E81+F81</f>
         <v/>
       </c>
@@ -8965,14 +8977,14 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="29" t="n">
+      <c r="A82" s="30" t="n">
         <v>38.23</v>
       </c>
-      <c r="B82" s="29">
+      <c r="B82" s="30">
         <f>A82-$B$12</f>
         <v/>
       </c>
-      <c r="C82" s="29">
+      <c r="C82" s="30">
         <f>MAX(0,A82-$B$6)</f>
         <v/>
       </c>
@@ -8988,7 +9000,7 @@
         <f>IF(A82&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A82&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A82,Stage_Storage!$A$11:$A$18,1))+(A82-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A82,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A82,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A82,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A82,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A82,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G82" s="31">
+      <c r="G82" s="32">
         <f>E82+F82</f>
         <v/>
       </c>
@@ -9010,14 +9022,14 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="29" t="n">
+      <c r="A83" s="30" t="n">
         <v>38.28</v>
       </c>
-      <c r="B83" s="29">
+      <c r="B83" s="30">
         <f>A83-$B$12</f>
         <v/>
       </c>
-      <c r="C83" s="29">
+      <c r="C83" s="30">
         <f>MAX(0,A83-$B$6)</f>
         <v/>
       </c>
@@ -9033,7 +9045,7 @@
         <f>IF(A83&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A83&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A83,Stage_Storage!$A$11:$A$18,1))+(A83-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A83,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A83,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A83,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A83,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A83,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G83" s="31">
+      <c r="G83" s="32">
         <f>E83+F83</f>
         <v/>
       </c>
@@ -9055,14 +9067,14 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="29" t="n">
+      <c r="A84" s="30" t="n">
         <v>38.33</v>
       </c>
-      <c r="B84" s="29">
+      <c r="B84" s="30">
         <f>A84-$B$12</f>
         <v/>
       </c>
-      <c r="C84" s="29">
+      <c r="C84" s="30">
         <f>MAX(0,A84-$B$6)</f>
         <v/>
       </c>
@@ -9078,7 +9090,7 @@
         <f>IF(A84&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A84&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A84,Stage_Storage!$A$11:$A$18,1))+(A84-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A84,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A84,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A84,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A84,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A84,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G84" s="31">
+      <c r="G84" s="32">
         <f>E84+F84</f>
         <v/>
       </c>
@@ -9100,14 +9112,14 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="29" t="n">
+      <c r="A85" s="30" t="n">
         <v>38.38</v>
       </c>
-      <c r="B85" s="29">
+      <c r="B85" s="30">
         <f>A85-$B$12</f>
         <v/>
       </c>
-      <c r="C85" s="29">
+      <c r="C85" s="30">
         <f>MAX(0,A85-$B$6)</f>
         <v/>
       </c>
@@ -9123,7 +9135,7 @@
         <f>IF(A85&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A85&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A85,Stage_Storage!$A$11:$A$18,1))+(A85-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A85,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A85,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A85,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A85,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A85,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G85" s="31">
+      <c r="G85" s="32">
         <f>E85+F85</f>
         <v/>
       </c>
@@ -9145,14 +9157,14 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="29" t="n">
+      <c r="A86" s="30" t="n">
         <v>38.43</v>
       </c>
-      <c r="B86" s="29">
+      <c r="B86" s="30">
         <f>A86-$B$12</f>
         <v/>
       </c>
-      <c r="C86" s="29">
+      <c r="C86" s="30">
         <f>MAX(0,A86-$B$6)</f>
         <v/>
       </c>
@@ -9168,7 +9180,7 @@
         <f>IF(A86&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A86&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A86,Stage_Storage!$A$11:$A$18,1))+(A86-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A86,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A86,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A86,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A86,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A86,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G86" s="31">
+      <c r="G86" s="32">
         <f>E86+F86</f>
         <v/>
       </c>
@@ -9190,14 +9202,14 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="29" t="n">
+      <c r="A87" s="30" t="n">
         <v>38.48</v>
       </c>
-      <c r="B87" s="29">
+      <c r="B87" s="30">
         <f>A87-$B$12</f>
         <v/>
       </c>
-      <c r="C87" s="29">
+      <c r="C87" s="30">
         <f>MAX(0,A87-$B$6)</f>
         <v/>
       </c>
@@ -9213,7 +9225,7 @@
         <f>IF(A87&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A87&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A87,Stage_Storage!$A$11:$A$18,1))+(A87-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A87,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A87,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A87,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A87,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A87,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G87" s="31">
+      <c r="G87" s="32">
         <f>E87+F87</f>
         <v/>
       </c>
@@ -9235,14 +9247,14 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="29" t="n">
+      <c r="A88" s="30" t="n">
         <v>38.53</v>
       </c>
-      <c r="B88" s="29">
+      <c r="B88" s="30">
         <f>A88-$B$12</f>
         <v/>
       </c>
-      <c r="C88" s="29">
+      <c r="C88" s="30">
         <f>MAX(0,A88-$B$6)</f>
         <v/>
       </c>
@@ -9258,7 +9270,7 @@
         <f>IF(A88&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A88&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A88,Stage_Storage!$A$11:$A$18,1))+(A88-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A88,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A88,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A88,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A88,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A88,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G88" s="31">
+      <c r="G88" s="32">
         <f>E88+F88</f>
         <v/>
       </c>
@@ -9280,14 +9292,14 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="29" t="n">
+      <c r="A89" s="30" t="n">
         <v>38.58</v>
       </c>
-      <c r="B89" s="29">
+      <c r="B89" s="30">
         <f>A89-$B$12</f>
         <v/>
       </c>
-      <c r="C89" s="29">
+      <c r="C89" s="30">
         <f>MAX(0,A89-$B$6)</f>
         <v/>
       </c>
@@ -9303,7 +9315,7 @@
         <f>IF(A89&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A89&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A89,Stage_Storage!$A$11:$A$18,1))+(A89-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A89,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A89,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A89,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A89,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A89,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G89" s="31">
+      <c r="G89" s="32">
         <f>E89+F89</f>
         <v/>
       </c>
@@ -9325,14 +9337,14 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="29" t="n">
+      <c r="A90" s="30" t="n">
         <v>38.63</v>
       </c>
-      <c r="B90" s="29">
+      <c r="B90" s="30">
         <f>A90-$B$12</f>
         <v/>
       </c>
-      <c r="C90" s="29">
+      <c r="C90" s="30">
         <f>MAX(0,A90-$B$6)</f>
         <v/>
       </c>
@@ -9348,7 +9360,7 @@
         <f>IF(A90&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A90&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A90,Stage_Storage!$A$11:$A$18,1))+(A90-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A90,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A90,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A90,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A90,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A90,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G90" s="31">
+      <c r="G90" s="32">
         <f>E90+F90</f>
         <v/>
       </c>
@@ -9370,14 +9382,14 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="29" t="n">
+      <c r="A91" s="30" t="n">
         <v>38.68</v>
       </c>
-      <c r="B91" s="29">
+      <c r="B91" s="30">
         <f>A91-$B$12</f>
         <v/>
       </c>
-      <c r="C91" s="29">
+      <c r="C91" s="30">
         <f>MAX(0,A91-$B$6)</f>
         <v/>
       </c>
@@ -9393,7 +9405,7 @@
         <f>IF(A91&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A91&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A91,Stage_Storage!$A$11:$A$18,1))+(A91-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A91,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A91,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A91,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A91,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A91,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G91" s="31">
+      <c r="G91" s="32">
         <f>E91+F91</f>
         <v/>
       </c>
@@ -9415,14 +9427,14 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="29" t="n">
+      <c r="A92" s="30" t="n">
         <v>38.73</v>
       </c>
-      <c r="B92" s="29">
+      <c r="B92" s="30">
         <f>A92-$B$12</f>
         <v/>
       </c>
-      <c r="C92" s="29">
+      <c r="C92" s="30">
         <f>MAX(0,A92-$B$6)</f>
         <v/>
       </c>
@@ -9438,7 +9450,7 @@
         <f>IF(A92&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A92&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A92,Stage_Storage!$A$11:$A$18,1))+(A92-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A92,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A92,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A92,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A92,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A92,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G92" s="31">
+      <c r="G92" s="32">
         <f>E92+F92</f>
         <v/>
       </c>
@@ -9460,14 +9472,14 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="29" t="n">
+      <c r="A93" s="30" t="n">
         <v>38.78</v>
       </c>
-      <c r="B93" s="29">
+      <c r="B93" s="30">
         <f>A93-$B$12</f>
         <v/>
       </c>
-      <c r="C93" s="29">
+      <c r="C93" s="30">
         <f>MAX(0,A93-$B$6)</f>
         <v/>
       </c>
@@ -9483,7 +9495,7 @@
         <f>IF(A93&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A93&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A93,Stage_Storage!$A$11:$A$18,1))+(A93-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A93,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A93,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A93,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A93,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A93,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G93" s="31">
+      <c r="G93" s="32">
         <f>E93+F93</f>
         <v/>
       </c>
@@ -9505,14 +9517,14 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="29" t="n">
+      <c r="A94" s="30" t="n">
         <v>38.83</v>
       </c>
-      <c r="B94" s="29">
+      <c r="B94" s="30">
         <f>A94-$B$12</f>
         <v/>
       </c>
-      <c r="C94" s="29">
+      <c r="C94" s="30">
         <f>MAX(0,A94-$B$6)</f>
         <v/>
       </c>
@@ -9528,7 +9540,7 @@
         <f>IF(A94&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A94&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A94,Stage_Storage!$A$11:$A$18,1))+(A94-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A94,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A94,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A94,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A94,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A94,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G94" s="31">
+      <c r="G94" s="32">
         <f>E94+F94</f>
         <v/>
       </c>
@@ -9550,14 +9562,14 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="29" t="n">
+      <c r="A95" s="30" t="n">
         <v>38.88</v>
       </c>
-      <c r="B95" s="29">
+      <c r="B95" s="30">
         <f>A95-$B$12</f>
         <v/>
       </c>
-      <c r="C95" s="29">
+      <c r="C95" s="30">
         <f>MAX(0,A95-$B$6)</f>
         <v/>
       </c>
@@ -9573,7 +9585,7 @@
         <f>IF(A95&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A95&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A95,Stage_Storage!$A$11:$A$18,1))+(A95-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A95,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A95,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A95,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A95,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A95,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G95" s="31">
+      <c r="G95" s="32">
         <f>E95+F95</f>
         <v/>
       </c>
@@ -9595,14 +9607,14 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="29" t="n">
+      <c r="A96" s="30" t="n">
         <v>38.93</v>
       </c>
-      <c r="B96" s="29">
+      <c r="B96" s="30">
         <f>A96-$B$12</f>
         <v/>
       </c>
-      <c r="C96" s="29">
+      <c r="C96" s="30">
         <f>MAX(0,A96-$B$6)</f>
         <v/>
       </c>
@@ -9618,7 +9630,7 @@
         <f>IF(A96&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A96&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A96,Stage_Storage!$A$11:$A$18,1))+(A96-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A96,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A96,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A96,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A96,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A96,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G96" s="31">
+      <c r="G96" s="32">
         <f>E96+F96</f>
         <v/>
       </c>
@@ -9640,14 +9652,14 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="29" t="n">
+      <c r="A97" s="30" t="n">
         <v>38.98</v>
       </c>
-      <c r="B97" s="29">
+      <c r="B97" s="30">
         <f>A97-$B$12</f>
         <v/>
       </c>
-      <c r="C97" s="29">
+      <c r="C97" s="30">
         <f>MAX(0,A97-$B$6)</f>
         <v/>
       </c>
@@ -9663,7 +9675,7 @@
         <f>IF(A97&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A97&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A97,Stage_Storage!$A$11:$A$18,1))+(A97-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A97,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A97,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A97,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A97,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A97,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G97" s="31">
+      <c r="G97" s="32">
         <f>E97+F97</f>
         <v/>
       </c>
@@ -9685,14 +9697,14 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="29" t="n">
+      <c r="A98" s="30" t="n">
         <v>39.03</v>
       </c>
-      <c r="B98" s="29">
+      <c r="B98" s="30">
         <f>A98-$B$12</f>
         <v/>
       </c>
-      <c r="C98" s="29">
+      <c r="C98" s="30">
         <f>MAX(0,A98-$B$6)</f>
         <v/>
       </c>
@@ -9708,7 +9720,7 @@
         <f>IF(A98&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A98&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A98,Stage_Storage!$A$11:$A$18,1))+(A98-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A98,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A98,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A98,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A98,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A98,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G98" s="31">
+      <c r="G98" s="32">
         <f>E98+F98</f>
         <v/>
       </c>
@@ -9730,14 +9742,14 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="29" t="n">
+      <c r="A99" s="30" t="n">
         <v>39.08</v>
       </c>
-      <c r="B99" s="29">
+      <c r="B99" s="30">
         <f>A99-$B$12</f>
         <v/>
       </c>
-      <c r="C99" s="29">
+      <c r="C99" s="30">
         <f>MAX(0,A99-$B$6)</f>
         <v/>
       </c>
@@ -9753,7 +9765,7 @@
         <f>IF(A99&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A99&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A99,Stage_Storage!$A$11:$A$18,1))+(A99-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A99,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A99,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A99,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A99,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A99,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G99" s="31">
+      <c r="G99" s="32">
         <f>E99+F99</f>
         <v/>
       </c>
@@ -9775,14 +9787,14 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="29" t="n">
+      <c r="A100" s="30" t="n">
         <v>39.13</v>
       </c>
-      <c r="B100" s="29">
+      <c r="B100" s="30">
         <f>A100-$B$12</f>
         <v/>
       </c>
-      <c r="C100" s="29">
+      <c r="C100" s="30">
         <f>MAX(0,A100-$B$6)</f>
         <v/>
       </c>
@@ -9798,7 +9810,7 @@
         <f>IF(A100&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A100&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A100,Stage_Storage!$A$11:$A$18,1))+(A100-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A100,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A100,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A100,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A100,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A100,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G100" s="31">
+      <c r="G100" s="32">
         <f>E100+F100</f>
         <v/>
       </c>
@@ -9820,14 +9832,14 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="29" t="n">
+      <c r="A101" s="30" t="n">
         <v>39.18</v>
       </c>
-      <c r="B101" s="29">
+      <c r="B101" s="30">
         <f>A101-$B$12</f>
         <v/>
       </c>
-      <c r="C101" s="29">
+      <c r="C101" s="30">
         <f>MAX(0,A101-$B$6)</f>
         <v/>
       </c>
@@ -9843,7 +9855,7 @@
         <f>IF(A101&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A101&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A101,Stage_Storage!$A$11:$A$18,1))+(A101-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A101,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A101,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A101,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A101,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A101,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G101" s="31">
+      <c r="G101" s="32">
         <f>E101+F101</f>
         <v/>
       </c>
@@ -9865,14 +9877,14 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="29" t="n">
+      <c r="A102" s="30" t="n">
         <v>39.23</v>
       </c>
-      <c r="B102" s="29">
+      <c r="B102" s="30">
         <f>A102-$B$12</f>
         <v/>
       </c>
-      <c r="C102" s="29">
+      <c r="C102" s="30">
         <f>MAX(0,A102-$B$6)</f>
         <v/>
       </c>
@@ -9888,7 +9900,7 @@
         <f>IF(A102&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A102&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A102,Stage_Storage!$A$11:$A$18,1))+(A102-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A102,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A102,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A102,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A102,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A102,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G102" s="31">
+      <c r="G102" s="32">
         <f>E102+F102</f>
         <v/>
       </c>
@@ -9910,14 +9922,14 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="29" t="n">
+      <c r="A103" s="30" t="n">
         <v>39.28</v>
       </c>
-      <c r="B103" s="29">
+      <c r="B103" s="30">
         <f>A103-$B$12</f>
         <v/>
       </c>
-      <c r="C103" s="29">
+      <c r="C103" s="30">
         <f>MAX(0,A103-$B$6)</f>
         <v/>
       </c>
@@ -9933,7 +9945,7 @@
         <f>IF(A103&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A103&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A103,Stage_Storage!$A$11:$A$18,1))+(A103-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A103,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A103,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A103,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A103,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A103,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G103" s="31">
+      <c r="G103" s="32">
         <f>E103+F103</f>
         <v/>
       </c>
@@ -9955,14 +9967,14 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="29" t="n">
+      <c r="A104" s="30" t="n">
         <v>39.33</v>
       </c>
-      <c r="B104" s="29">
+      <c r="B104" s="30">
         <f>A104-$B$12</f>
         <v/>
       </c>
-      <c r="C104" s="29">
+      <c r="C104" s="30">
         <f>MAX(0,A104-$B$6)</f>
         <v/>
       </c>
@@ -9978,7 +9990,7 @@
         <f>IF(A104&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A104&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A104,Stage_Storage!$A$11:$A$18,1))+(A104-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A104,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A104,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A104,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A104,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A104,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G104" s="31">
+      <c r="G104" s="32">
         <f>E104+F104</f>
         <v/>
       </c>
@@ -10000,14 +10012,14 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="29" t="n">
+      <c r="A105" s="30" t="n">
         <v>39.38</v>
       </c>
-      <c r="B105" s="29">
+      <c r="B105" s="30">
         <f>A105-$B$12</f>
         <v/>
       </c>
-      <c r="C105" s="29">
+      <c r="C105" s="30">
         <f>MAX(0,A105-$B$6)</f>
         <v/>
       </c>
@@ -10023,7 +10035,7 @@
         <f>IF(A105&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A105&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A105,Stage_Storage!$A$11:$A$18,1))+(A105-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A105,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A105,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A105,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A105,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A105,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G105" s="31">
+      <c r="G105" s="32">
         <f>E105+F105</f>
         <v/>
       </c>
@@ -10045,14 +10057,14 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="29" t="n">
+      <c r="A106" s="30" t="n">
         <v>39.43</v>
       </c>
-      <c r="B106" s="29">
+      <c r="B106" s="30">
         <f>A106-$B$12</f>
         <v/>
       </c>
-      <c r="C106" s="29">
+      <c r="C106" s="30">
         <f>MAX(0,A106-$B$6)</f>
         <v/>
       </c>
@@ -10068,7 +10080,7 @@
         <f>IF(A106&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A106&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A106,Stage_Storage!$A$11:$A$18,1))+(A106-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A106,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A106,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A106,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A106,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A106,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G106" s="31">
+      <c r="G106" s="32">
         <f>E106+F106</f>
         <v/>
       </c>
@@ -10090,14 +10102,14 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="29" t="n">
+      <c r="A107" s="30" t="n">
         <v>39.48</v>
       </c>
-      <c r="B107" s="29">
+      <c r="B107" s="30">
         <f>A107-$B$12</f>
         <v/>
       </c>
-      <c r="C107" s="29">
+      <c r="C107" s="30">
         <f>MAX(0,A107-$B$6)</f>
         <v/>
       </c>
@@ -10113,7 +10125,7 @@
         <f>IF(A107&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A107&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A107,Stage_Storage!$A$11:$A$18,1))+(A107-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A107,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A107,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A107,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A107,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A107,Stage_Storage!$A$11:$A$18,1)))))</f>
         <v/>
       </c>
-      <c r="G107" s="31">
+      <c r="G107" s="32">
         <f>E107+F107</f>
         <v/>
       </c>
@@ -10169,7 +10181,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="37" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>À chaque pas: WSE lu sur Compose_900!V_total → Qout sur Compose_900. ΔV = (Qin_moy − Qout)×Δt. Si V≈0, Qout = MIN(Qin, Q_plein).</t>
         </is>
@@ -10182,7 +10194,7 @@
           <t>Q_plein réf. (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="38">
+      <c r="B5" s="39">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -10193,7 +10205,7 @@
           <t>Crest (m)</t>
         </is>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="39">
         <f>Parametres!B27</f>
         <v/>
       </c>
@@ -10204,7 +10216,7 @@
           <t>Vmax_C (m³)</t>
         </is>
       </c>
-      <c r="B7" s="28">
+      <c r="B7" s="29">
         <f>MAX(F12:F24)</f>
         <v/>
       </c>
@@ -10288,7 +10300,7 @@
       <c r="E12" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="31" t="n">
+      <c r="F12" s="32" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -10318,7 +10330,7 @@
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="32">
         <f>MAX(0,F12+(0.5*(B12+B13)-D13)*E13)</f>
         <v/>
       </c>
@@ -10348,7 +10360,7 @@
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="32">
         <f>MAX(0,F13+(0.5*(B13+B14)-D14)*E14)</f>
         <v/>
       </c>
@@ -10378,7 +10390,7 @@
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="32">
         <f>MAX(0,F14+(0.5*(B14+B15)-D15)*E15)</f>
         <v/>
       </c>
@@ -10408,7 +10420,7 @@
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="32">
         <f>MAX(0,F15+(0.5*(B15+B16)-D16)*E16)</f>
         <v/>
       </c>
@@ -10438,7 +10450,7 @@
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="F17" s="31">
+      <c r="F17" s="32">
         <f>MAX(0,F16+(0.5*(B16+B17)-D17)*E17)</f>
         <v/>
       </c>
@@ -10468,7 +10480,7 @@
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="F18" s="31">
+      <c r="F18" s="32">
         <f>MAX(0,F17+(0.5*(B17+B18)-D18)*E18)</f>
         <v/>
       </c>
@@ -10498,7 +10510,7 @@
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="F19" s="31">
+      <c r="F19" s="32">
         <f>MAX(0,F18+(0.5*(B18+B19)-D19)*E19)</f>
         <v/>
       </c>
@@ -10528,7 +10540,7 @@
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="F20" s="31">
+      <c r="F20" s="32">
         <f>MAX(0,F19+(0.5*(B19+B20)-D20)*E20)</f>
         <v/>
       </c>
@@ -10558,7 +10570,7 @@
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="F21" s="31">
+      <c r="F21" s="32">
         <f>MAX(0,F20+(0.5*(B20+B21)-D21)*E21)</f>
         <v/>
       </c>
@@ -10588,7 +10600,7 @@
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="F22" s="31">
+      <c r="F22" s="32">
         <f>MAX(0,F21+(0.5*(B21+B22)-D22)*E22)</f>
         <v/>
       </c>
@@ -10618,7 +10630,7 @@
         <f>(A23-A22)*60</f>
         <v/>
       </c>
-      <c r="F23" s="31">
+      <c r="F23" s="32">
         <f>MAX(0,F22+(0.5*(B22+B23)-D23)*E23)</f>
         <v/>
       </c>
@@ -10648,7 +10660,7 @@
         <f>(A24-A23)*60</f>
         <v/>
       </c>
-      <c r="F24" s="31">
+      <c r="F24" s="32">
         <f>MAX(0,F23+(0.5*(B23+B24)-D24)*E24)</f>
         <v/>
       </c>
@@ -10706,7 +10718,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>V_pas (m³) = (A_basse + A_haute) / 2 × (WSE_haute − WSE_basse)</t>
         </is>
@@ -10752,7 +10764,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="n">
+      <c r="A11" s="30" t="n">
         <v>34.88</v>
       </c>
       <c r="B11" s="17" t="n">
@@ -10774,13 +10786,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="n">
+      <c r="A12" s="30" t="n">
         <v>35.5</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>80</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="30">
         <f>A12-A11</f>
         <v/>
       </c>
@@ -10788,7 +10800,7 @@
         <f>0.5*(B11+B12)*C12</f>
         <v/>
       </c>
-      <c r="E12" s="31">
+      <c r="E12" s="32">
         <f>E11+D12</f>
         <v/>
       </c>
@@ -10799,13 +10811,13 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="n">
+      <c r="A13" s="30" t="n">
         <v>36</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>180</v>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="30">
         <f>A13-A12</f>
         <v/>
       </c>
@@ -10813,7 +10825,7 @@
         <f>0.5*(B12+B13)*C13</f>
         <v/>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="32">
         <f>E12+D13</f>
         <v/>
       </c>
@@ -10824,13 +10836,13 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="n">
+      <c r="A14" s="30" t="n">
         <v>36.5</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>320</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="30">
         <f>A14-A13</f>
         <v/>
       </c>
@@ -10838,7 +10850,7 @@
         <f>0.5*(B13+B14)*C14</f>
         <v/>
       </c>
-      <c r="E14" s="31">
+      <c r="E14" s="32">
         <f>E13+D14</f>
         <v/>
       </c>
@@ -10849,13 +10861,13 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="n">
+      <c r="A15" s="30" t="n">
         <v>37</v>
       </c>
       <c r="B15" s="17" t="n">
         <v>480</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="30">
         <f>A15-A14</f>
         <v/>
       </c>
@@ -10863,7 +10875,7 @@
         <f>0.5*(B14+B15)*C15</f>
         <v/>
       </c>
-      <c r="E15" s="31">
+      <c r="E15" s="32">
         <f>E14+D15</f>
         <v/>
       </c>
@@ -10874,21 +10886,21 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="n">
+      <c r="A16" s="37" t="n">
         <v>37.28</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>543</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="37">
         <f>A16-A15</f>
         <v/>
       </c>
-      <c r="D16" s="39">
+      <c r="D16" s="40">
         <f>0.5*(B15+B16)*C16</f>
         <v/>
       </c>
-      <c r="E16" s="39">
+      <c r="E16" s="40">
         <f>E15+D16</f>
         <v/>
       </c>
@@ -10899,13 +10911,13 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="n">
+      <c r="A17" s="30" t="n">
         <v>37.5</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>700</v>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="30">
         <f>A17-A16</f>
         <v/>
       </c>
@@ -10913,7 +10925,7 @@
         <f>0.5*(B16+B17)*C17</f>
         <v/>
       </c>
-      <c r="E17" s="31">
+      <c r="E17" s="32">
         <f>E16+D17</f>
         <v/>
       </c>
@@ -10924,13 +10936,13 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="n">
+      <c r="A18" s="30" t="n">
         <v>39.5</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>1932</v>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="30">
         <f>A18-A17</f>
         <v/>
       </c>
@@ -10938,7 +10950,7 @@
         <f>0.5*(B17+B18)*C18</f>
         <v/>
       </c>
-      <c r="E18" s="31">
+      <c r="E18" s="32">
         <f>E17+D18</f>
         <v/>
       </c>
@@ -10965,7 +10977,7 @@
           <t>WSEmax_A (m)</t>
         </is>
       </c>
-      <c r="B22" s="40">
+      <c r="B22" s="41">
         <f>Parametres!B39</f>
         <v/>
       </c>
@@ -10987,7 +10999,7 @@
           <t>WSEmax_B (m)</t>
         </is>
       </c>
-      <c r="B24" s="40">
+      <c r="B24" s="41">
         <f>Parametres!B45</f>
         <v/>
       </c>
@@ -11018,7 +11030,7 @@
           <t>V disponible à 37.28 m (m³)</t>
         </is>
       </c>
-      <c r="B26" s="41">
+      <c r="B26" s="42">
         <f>E16</f>
         <v/>
       </c>
@@ -11036,7 +11048,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="37" t="inlineStr">
+      <c r="A29" s="38" t="inlineStr">
         <is>
           <t>Exemple: si Vmax_A = 5609 m³ et V(37.28)≈558 m³, alors WSEmax_A est au-dessus de 37.28 m (la table ira vers 39.5 m ou 'Hors table'). Affinez en entrant les vraies surfaces aux cotes intermédiaires (jaune). Méthode C: voir Parametres B49–B52 et Calcul_C (fossé inclus).</t>
         </is>
@@ -11069,7 +11081,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>Où sont les fichiers HY-8 / capacité ?</t>
         </is>

</xml_diff>

<commit_message>
Replace Stage_Storage with survey areas; clarify B24 is Method B only
Use the real levé surface table (34.88→40.00). Relabel Parametres B24 so
it is not mistaken for a second pond — it only drives H≈V/A in Method B.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -1861,7 +1861,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aire_bassin_m2</t>
+          <t>Aire_constante_B (m²) — PAS le levé</t>
         </is>
       </c>
       <c r="B24" s="17" t="n">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Aire plan d'eau approx. pour H = V/A (Méthode B seulement)</t>
+          <t>Raccourci Méthode B seulement: H≈V/B24 pour lire Q=f(H). Ce n'est PAS un 2e bassin. Le vrai étang = feuille Stage_Storage (surfaces vs WSE).</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="B39" s="22">
-        <f>IF(B36&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B36&gt;=Stage_Storage!E18,"Hors table (&gt;=39.5 m — étendre levé)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1))+(B36-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))))</f>
+        <f>IF(B36&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B36&gt;=Stage_Storage!E18,"Hors table (&gt;=40.0 m — étendre levé)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1))+(B36-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))))</f>
         <v/>
       </c>
       <c r="C39" t="inlineStr">
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="B45" s="22">
-        <f>IF(B43&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B43&gt;=Stage_Storage!E18,"Hors table (&gt;=39.5 m — étendre levé)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1))+(B43-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)))))</f>
+        <f>IF(B43&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B43&gt;=Stage_Storage!E18,"Hors table (&gt;=40.0 m — étendre levé)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1))+(B43-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B43,Stage_Storage!$E$11:$E$18,1)))))</f>
         <v/>
       </c>
       <c r="C45" t="inlineStr">
@@ -5321,7 +5321,7 @@
     <row r="2">
       <c r="A2" s="39" t="inlineStr">
         <is>
-          <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. La courbe Courbe_QH_900 est en formules live (changer n/L/entrée/TW).</t>
+          <t>H = V / Aire_constante (Parametres!B24) — raccourci, PAS le levé Stage_Storage. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. Après routage, WSEmax_B réel est lu sur Stage_Storage via Vmax_B (Parametres B45).</t>
         </is>
       </c>
     </row>
@@ -10722,7 +10722,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>PROCÉDURE (dans CE fichier): 1) Routage → Vmax_A / Vmax_B / Vmax_C sur Parametres. 2) Cette feuille = V_pond vs WSE (levé seul). 3) Parametres!B39 = WSEmax_A; B45 = WSEmax_B (levé). 4) Méthode C: V_pond + V_ditch et WSEmax_C sont sur Compose_900 / Calcul_C (B51). Remplacez les surfaces jaunes; 543 m² @ 37.28 et 1932 m² @ 39.5 sont vos mesures.</t>
+          <t>PROCÉDURE (dans CE fichier): 1) Routage → Vmax_A / Vmax_B / Vmax_C sur Parametres. 2) Cette feuille = V_pond vs WSE (levé topographique — le vrai bassin). 3) Parametres!B39 = WSEmax_A; B45 = WSEmax_B (lus sur CE tableau). 4) Méthode C: V_pond + V_ditch et WSEmax_C sur Compose_900 / Calcul_C (B51). 5) Parametres!B24 (2500 m²) n'est PAS ici: c'est seulement le raccourci H=V/A de Méthode B. Surfaces ci-dessous = votre levé (pas des placeholders).</t>
         </is>
       </c>
     </row>
@@ -10799,7 +10799,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Radier Ø900 — départ</t>
+          <t>Fond bassin / radier Ø900</t>
         </is>
       </c>
     </row>
@@ -10808,7 +10808,7 @@
         <v>35.5</v>
       </c>
       <c r="B12" s="17" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C12" s="31">
         <f>A12-A11</f>
@@ -10824,16 +10824,16 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer par levé</t>
+          <t>Levé</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="31" t="n">
-        <v>36</v>
+        <v>36.01</v>
       </c>
       <c r="B13" s="17" t="n">
-        <v>180</v>
+        <v>419</v>
       </c>
       <c r="C13" s="31">
         <f>A13-A12</f>
@@ -10849,7 +10849,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer par levé</t>
+          <t>Levé</t>
         </is>
       </c>
     </row>
@@ -10858,7 +10858,7 @@
         <v>36.5</v>
       </c>
       <c r="B14" s="17" t="n">
-        <v>320</v>
+        <v>480</v>
       </c>
       <c r="C14" s="31">
         <f>A14-A13</f>
@@ -10874,7 +10874,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer par levé</t>
+          <t>Levé</t>
         </is>
       </c>
     </row>
@@ -10883,7 +10883,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="17" t="n">
-        <v>480</v>
+        <v>720</v>
       </c>
       <c r="C15" s="31">
         <f>A15-A14</f>
@@ -10899,7 +10899,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer par levé</t>
+          <t>Levé</t>
         </is>
       </c>
     </row>
@@ -10908,7 +10908,7 @@
         <v>37.28</v>
       </c>
       <c r="B16" s="17" t="n">
-        <v>543</v>
+        <v>2198</v>
       </c>
       <c r="C16" s="38">
         <f>A16-A15</f>
@@ -10924,16 +10924,16 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>LIMITE PATRON (+1.5 m crown) — votre levé</t>
+          <t>LIMITE PATRON (+1.5 m crown) — levé</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="31" t="n">
-        <v>37.5</v>
+        <v>37.4</v>
       </c>
       <c r="B17" s="17" t="n">
-        <v>700</v>
+        <v>1516</v>
       </c>
       <c r="C17" s="31">
         <f>A17-A16</f>
@@ -10949,16 +10949,16 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer par levé</t>
+          <t>Levé (A↓ vs 37.28 — vérifier si voulu)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="31" t="n">
-        <v>39.5</v>
+        <v>40</v>
       </c>
       <c r="B18" s="17" t="n">
-        <v>1932</v>
+        <v>3746</v>
       </c>
       <c r="C18" s="31">
         <f>A18-A17</f>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Votre levé 1932 m² — niveau optionnel plus haut</t>
+          <t>Levé — sommet table</t>
         </is>
       </c>
     </row>
@@ -11068,7 +11068,7 @@
     <row r="29">
       <c r="A29" s="39" t="inlineStr">
         <is>
-          <t>Exemple: si Vmax_A = 5609 m³ et V(37.28)≈558 m³, alors WSEmax_A est au-dessus de 37.28 m (la table ira vers 39.5 m ou 'Hors table'). Affinez en entrant les vraies surfaces aux cotes intermédiaires (jaune). Méthode C: voir Parametres B49–B52 et Calcul_C (fossé inclus).</t>
+          <t>Exemple: si Vmax_A &gt; V_cumul @ 37.28 (colonne E, ligne orange), alors WSEmax_A &gt; 37.28 m (la table monte vers 37.40 / 40.00 ou 'Hors table'). Jaune = surfaces du levé (éditables). Méthode C: Parametres B49–B52 et Calcul_C (fossé inclus). Note: A(37.40)=1516 &lt; A(37.28)=2198 — inhabituel; confirmer sur plan.</t>
         </is>
       </c>
     </row>

</xml_diff>